<commit_message>
Update as_building drawing v1.11
</commit_message>
<xml_diff>
--- a/vor_lublino.xlsx
+++ b/vor_lublino.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="60">
   <si>
     <t>Штукатурка цементным составом толщиной 16‐20 мм</t>
   </si>
@@ -190,6 +190,12 @@
   </si>
   <si>
     <t>1.026</t>
+  </si>
+  <si>
+    <t>717.47 п.м</t>
+  </si>
+  <si>
+    <t>Сетка штукатурная стеклопакетная 10х10 мм</t>
   </si>
 </sst>
 </file>
@@ -895,7 +901,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A3:G127"/>
+  <dimension ref="A3:G133"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.7109375" style="35" customWidth="1"/>
@@ -950,7 +956,7 @@
         <v>2</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="D6" s="16">
         <f>D5</f>
@@ -1014,7 +1020,7 @@
         <v>2</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="D13" s="16">
         <f>D12</f>
@@ -1078,7 +1084,7 @@
         <v>2</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="D20" s="16">
         <f>D19</f>
@@ -1142,7 +1148,7 @@
         <v>2</v>
       </c>
       <c r="C27" s="15" t="s">
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="D27" s="16">
         <f>D26</f>
@@ -1206,7 +1212,7 @@
         <v>2</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="D34" s="16">
         <f>D33</f>
@@ -1270,7 +1276,7 @@
         <v>2</v>
       </c>
       <c r="C41" s="15" t="s">
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="D41" s="16">
         <f>D40</f>
@@ -1334,7 +1340,7 @@
         <v>2</v>
       </c>
       <c r="C48" s="15" t="s">
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="D48" s="16">
         <f>D47</f>
@@ -1398,7 +1404,7 @@
         <v>2</v>
       </c>
       <c r="C55" s="15" t="s">
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="D55" s="16">
         <f>D54</f>
@@ -1462,7 +1468,7 @@
         <v>2</v>
       </c>
       <c r="C62" s="15" t="s">
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="D62" s="16">
         <f>D61</f>
@@ -1526,7 +1532,7 @@
         <v>2</v>
       </c>
       <c r="C69" s="15" t="s">
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="D69" s="16">
         <f>D68</f>
@@ -1590,7 +1596,7 @@
         <v>2</v>
       </c>
       <c r="C76" s="15" t="s">
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="D76" s="16">
         <f>D75</f>
@@ -1654,7 +1660,7 @@
         <v>2</v>
       </c>
       <c r="C83" s="15" t="s">
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="D83" s="16">
         <f>D82</f>
@@ -1718,7 +1724,7 @@
         <v>2</v>
       </c>
       <c r="C90" s="15" t="s">
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="D90" s="16">
         <f>D89</f>
@@ -1770,11 +1776,11 @@
         <v>1</v>
       </c>
       <c r="D96" s="16">
-        <v>260.33</v>
+        <v>260.64999999999998</v>
       </c>
       <c r="G96" s="37">
         <f>D96</f>
-        <v>260.33</v>
+        <v>260.64999999999998</v>
       </c>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.2">
@@ -1782,11 +1788,11 @@
         <v>2</v>
       </c>
       <c r="C97" s="15" t="s">
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="D97" s="16">
         <f>D96</f>
-        <v>260.33</v>
+        <v>260.64999999999998</v>
       </c>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.2">
@@ -1846,7 +1852,7 @@
         <v>2</v>
       </c>
       <c r="C104" s="15" t="s">
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="D104" s="16">
         <f>D103</f>
@@ -1897,10 +1903,12 @@
       <c r="C110" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="D110" s="16"/>
+      <c r="D110" s="16">
+        <v>75.8</v>
+      </c>
       <c r="G110" s="37">
         <f>D110</f>
-        <v>0</v>
+        <v>75.8</v>
       </c>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.2">
@@ -1908,11 +1916,11 @@
         <v>2</v>
       </c>
       <c r="C111" s="15" t="s">
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="D111" s="16">
         <f>D110</f>
-        <v>0</v>
+        <v>75.8</v>
       </c>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.2">
@@ -1972,7 +1980,7 @@
         <v>2</v>
       </c>
       <c r="C118" s="15" t="s">
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="D118" s="16">
         <f>D117</f>
@@ -2024,11 +2032,11 @@
         <v>1</v>
       </c>
       <c r="D124" s="16">
-        <v>405.57</v>
+        <v>405.22</v>
       </c>
       <c r="G124" s="37">
         <f>D124</f>
-        <v>405.57</v>
+        <v>405.22</v>
       </c>
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.2">
@@ -2036,11 +2044,11 @@
         <v>2</v>
       </c>
       <c r="C125" s="15" t="s">
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="D125" s="16">
         <f>D124</f>
-        <v>405.57</v>
+        <v>405.22</v>
       </c>
     </row>
     <row r="126" spans="1:7" x14ac:dyDescent="0.2">
@@ -2058,6 +2066,63 @@
       <c r="B127" s="18"/>
       <c r="C127" s="19"/>
       <c r="D127" s="20"/>
+    </row>
+    <row r="129" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B129" s="9"/>
+      <c r="C129" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="D129" s="11"/>
+    </row>
+    <row r="130" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B130" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="C130" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D130" s="16" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="131" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B131" s="14">
+        <v>1</v>
+      </c>
+      <c r="C131" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="D131" s="16">
+        <f>G131</f>
+        <v>2606.7700000000004</v>
+      </c>
+      <c r="G131" s="13">
+        <f>SUM(G1:G126)</f>
+        <v>2606.7700000000004</v>
+      </c>
+    </row>
+    <row r="132" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B132" s="14">
+        <v>2</v>
+      </c>
+      <c r="C132" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D132" s="16">
+        <f>D131</f>
+        <v>2606.7700000000004</v>
+      </c>
+    </row>
+    <row r="133" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B133" s="14">
+        <v>3</v>
+      </c>
+      <c r="C133" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="D133" s="16" t="s">
+        <v>58</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2411,7 +2476,7 @@
       </c>
       <c r="E28" s="12"/>
     </row>
-    <row r="29" spans="1:7" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:7" s="13" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A29" s="35"/>
       <c r="B29" s="14">
         <v>6</v>
@@ -2536,7 +2601,7 @@
       </c>
       <c r="E39" s="12"/>
     </row>
-    <row r="40" spans="1:5" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:5" s="13" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A40" s="35"/>
       <c r="B40" s="14">
         <v>6</v>
@@ -2654,7 +2719,7 @@
       </c>
       <c r="E49" s="12"/>
     </row>
-    <row r="50" spans="1:5" s="26" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:5" s="26" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A50" s="36"/>
       <c r="B50" s="14">
         <v>6</v>
@@ -2774,7 +2839,7 @@
       </c>
       <c r="E59" s="30"/>
     </row>
-    <row r="60" spans="1:5" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:5" s="13" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A60" s="35"/>
       <c r="B60" s="14">
         <v>6</v>

</xml_diff>

<commit_message>
Update as_building drawing v1.13 lublino
Доделал потолок в люблино
</commit_message>
<xml_diff>
--- a/vor_lublino.xlsx
+++ b/vor_lublino.xlsx
@@ -4,20 +4,22 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="23265" yWindow="5565" windowWidth="5535" windowHeight="6105" activeTab="1"/>
+    <workbookView xWindow="23265" yWindow="5565" windowWidth="5535" windowHeight="6105" firstSheet="2" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Пример" sheetId="1" r:id="rId1"/>
     <sheet name="стены штукатурка" sheetId="2" r:id="rId2"/>
     <sheet name="Стены итог шт" sheetId="4" r:id="rId3"/>
     <sheet name="Стены шпаклевка" sheetId="3" r:id="rId4"/>
+    <sheet name="Потолок" sheetId="5" r:id="rId5"/>
+    <sheet name="Потолок итог шт (2)" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="145621"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="93">
   <si>
     <t>Штукатурка цементным составом толщиной 16‐20 мм</t>
   </si>
@@ -248,13 +250,61 @@
   </si>
   <si>
     <t>Грунтовка универсальный ЛАСТИМИН / LP-51 А</t>
+  </si>
+  <si>
+    <t>1.053, 1.054</t>
+  </si>
+  <si>
+    <t>Шлифование бетонных поверхностей</t>
+  </si>
+  <si>
+    <t>1.034-1.039</t>
+  </si>
+  <si>
+    <t>Шпатлевка гипсовая белая</t>
+  </si>
+  <si>
+    <t>Подготовка поверхности потолка СКБ</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>2.1</t>
+  </si>
+  <si>
+    <t>2.2</t>
+  </si>
+  <si>
+    <t>2.3</t>
+  </si>
+  <si>
+    <t>2.4</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>3.1</t>
+  </si>
+  <si>
+    <t>3.2</t>
+  </si>
+  <si>
+    <t>Ведомость используемых материалов</t>
+  </si>
+  <si>
+    <t>Грунт универсальный ЛАСТИМИН</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -292,6 +342,35 @@
       <family val="2"/>
       <charset val="204"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="ГОСТ тип А"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="ГОСТ тип А"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="ГОСТ тип А"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="ГОСТ тип А"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -301,7 +380,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="37">
+  <borders count="40">
     <border>
       <left/>
       <right/>
@@ -793,11 +872,56 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color theme="0"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="0"/>
+      </left>
+      <right style="medium">
+        <color theme="0"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="0"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="99">
+  <cellXfs count="183">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1077,6 +1201,232 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -3751,4 +4101,1141 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B2:H65"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="152"/>
+    <col min="2" max="2" width="7" style="152" customWidth="1"/>
+    <col min="3" max="3" width="10" style="152" customWidth="1"/>
+    <col min="4" max="4" width="56.85546875" style="152" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.28515625" style="152" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" style="152" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="152"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:8" s="152" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="2:8" s="105" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="153"/>
+      <c r="C3" s="154"/>
+      <c r="D3" s="155" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="156"/>
+      <c r="F3" s="157"/>
+      <c r="G3" s="158"/>
+    </row>
+    <row r="4" spans="2:8" s="105" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="159" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="160" t="s">
+        <v>58</v>
+      </c>
+      <c r="D4" s="161" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="135" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="157"/>
+      <c r="G4" s="158"/>
+    </row>
+    <row r="5" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="162">
+        <v>1</v>
+      </c>
+      <c r="C5" s="163" t="s">
+        <v>54</v>
+      </c>
+      <c r="D5" s="164" t="s">
+        <v>78</v>
+      </c>
+      <c r="E5" s="165">
+        <v>336.4</v>
+      </c>
+      <c r="F5" s="157"/>
+      <c r="G5" s="158"/>
+    </row>
+    <row r="6" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="166"/>
+      <c r="C6" s="167"/>
+      <c r="D6" s="140" t="s">
+        <v>1</v>
+      </c>
+      <c r="E6" s="126">
+        <v>30.2</v>
+      </c>
+      <c r="F6" s="157"/>
+      <c r="G6" s="158"/>
+      <c r="H6" s="158">
+        <f>E6</f>
+        <v>30.2</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="166"/>
+      <c r="C7" s="167"/>
+      <c r="D7" s="140" t="s">
+        <v>57</v>
+      </c>
+      <c r="E7" s="126">
+        <f>E6</f>
+        <v>30.2</v>
+      </c>
+      <c r="F7" s="157"/>
+      <c r="G7" s="158"/>
+    </row>
+    <row r="8" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="166"/>
+      <c r="C8" s="167"/>
+      <c r="D8" s="168" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" s="169" t="str">
+        <f>TEXT(G8, "0.00") &amp; " п.м"</f>
+        <v>60.41 п.м</v>
+      </c>
+      <c r="F8" s="157"/>
+      <c r="G8" s="158">
+        <v>60.41</v>
+      </c>
+    </row>
+    <row r="9" spans="2:8" s="105" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="170"/>
+      <c r="C9" s="171"/>
+      <c r="D9" s="172" t="s">
+        <v>81</v>
+      </c>
+      <c r="E9" s="130">
+        <f>E5</f>
+        <v>336.4</v>
+      </c>
+      <c r="F9" s="157"/>
+      <c r="G9" s="158"/>
+    </row>
+    <row r="10" spans="2:8" s="105" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="153"/>
+      <c r="C10" s="154"/>
+      <c r="D10" s="155" t="s">
+        <v>9</v>
+      </c>
+      <c r="E10" s="156"/>
+      <c r="F10" s="157"/>
+      <c r="G10" s="158"/>
+    </row>
+    <row r="11" spans="2:8" s="105" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="159" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" s="160" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" s="161" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" s="135" t="s">
+        <v>28</v>
+      </c>
+      <c r="F11" s="157"/>
+      <c r="G11" s="158"/>
+    </row>
+    <row r="12" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="173">
+        <v>2</v>
+      </c>
+      <c r="C12" s="174" t="s">
+        <v>77</v>
+      </c>
+      <c r="D12" s="175" t="s">
+        <v>78</v>
+      </c>
+      <c r="E12" s="123">
+        <v>543.35</v>
+      </c>
+      <c r="F12" s="157"/>
+      <c r="G12" s="158"/>
+    </row>
+    <row r="13" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="166"/>
+      <c r="C13" s="167"/>
+      <c r="D13" s="140" t="s">
+        <v>1</v>
+      </c>
+      <c r="E13" s="126">
+        <v>28.32</v>
+      </c>
+      <c r="F13" s="157"/>
+      <c r="G13" s="158"/>
+      <c r="H13" s="158">
+        <f>E13</f>
+        <v>28.32</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="166"/>
+      <c r="C14" s="167"/>
+      <c r="D14" s="140" t="s">
+        <v>57</v>
+      </c>
+      <c r="E14" s="126">
+        <f>E13</f>
+        <v>28.32</v>
+      </c>
+      <c r="F14" s="157"/>
+      <c r="G14" s="158"/>
+    </row>
+    <row r="15" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="166"/>
+      <c r="C15" s="167"/>
+      <c r="D15" s="168" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" s="169" t="str">
+        <f>TEXT(G15, "0.00") &amp; " п.м"</f>
+        <v>51.28 п.м</v>
+      </c>
+      <c r="F15" s="157"/>
+      <c r="G15" s="158">
+        <v>51.28</v>
+      </c>
+    </row>
+    <row r="16" spans="2:8" s="105" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="170"/>
+      <c r="C16" s="171"/>
+      <c r="D16" s="172" t="s">
+        <v>81</v>
+      </c>
+      <c r="E16" s="130">
+        <f>E12</f>
+        <v>543.35</v>
+      </c>
+      <c r="F16" s="157"/>
+      <c r="G16" s="158"/>
+    </row>
+    <row r="17" spans="2:7" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="106"/>
+      <c r="C17" s="176"/>
+      <c r="D17" s="177"/>
+      <c r="E17" s="178"/>
+      <c r="F17" s="157"/>
+      <c r="G17" s="158"/>
+    </row>
+    <row r="18" spans="2:7" s="105" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="106"/>
+      <c r="C18" s="176"/>
+      <c r="D18" s="177"/>
+      <c r="E18" s="178"/>
+      <c r="F18" s="157"/>
+      <c r="G18" s="158"/>
+    </row>
+    <row r="19" spans="2:7" s="105" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="153"/>
+      <c r="C19" s="154"/>
+      <c r="D19" s="155" t="s">
+        <v>9</v>
+      </c>
+      <c r="E19" s="156"/>
+      <c r="F19" s="157"/>
+      <c r="G19" s="158"/>
+    </row>
+    <row r="20" spans="2:7" s="105" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="159" t="s">
+        <v>6</v>
+      </c>
+      <c r="C20" s="160" t="s">
+        <v>58</v>
+      </c>
+      <c r="D20" s="161" t="s">
+        <v>7</v>
+      </c>
+      <c r="E20" s="135" t="s">
+        <v>28</v>
+      </c>
+      <c r="F20" s="157"/>
+      <c r="G20" s="158"/>
+    </row>
+    <row r="21" spans="2:7" s="105" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="B21" s="173">
+        <v>3</v>
+      </c>
+      <c r="C21" s="179" t="s">
+        <v>79</v>
+      </c>
+      <c r="D21" s="175" t="s">
+        <v>78</v>
+      </c>
+      <c r="E21" s="123">
+        <v>196.34</v>
+      </c>
+      <c r="F21" s="157"/>
+      <c r="G21" s="158"/>
+    </row>
+    <row r="22" spans="2:7" s="105" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="170"/>
+      <c r="C22" s="180"/>
+      <c r="D22" s="172" t="s">
+        <v>81</v>
+      </c>
+      <c r="E22" s="130">
+        <f>E21</f>
+        <v>196.34</v>
+      </c>
+      <c r="F22" s="157"/>
+      <c r="G22" s="158"/>
+    </row>
+    <row r="23" spans="2:7" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="106"/>
+      <c r="C23" s="176"/>
+      <c r="D23" s="177"/>
+      <c r="E23" s="178"/>
+      <c r="F23" s="157"/>
+      <c r="G23" s="158"/>
+    </row>
+    <row r="24" spans="2:7" s="105" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="106"/>
+      <c r="C24" s="176"/>
+      <c r="D24" s="177"/>
+      <c r="E24" s="178"/>
+      <c r="F24" s="157"/>
+      <c r="G24" s="158"/>
+    </row>
+    <row r="25" spans="2:7" s="105" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="153"/>
+      <c r="C25" s="154"/>
+      <c r="D25" s="155" t="s">
+        <v>9</v>
+      </c>
+      <c r="E25" s="156"/>
+      <c r="F25" s="157"/>
+      <c r="G25" s="158"/>
+    </row>
+    <row r="26" spans="2:7" s="105" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="159" t="s">
+        <v>6</v>
+      </c>
+      <c r="C26" s="160" t="s">
+        <v>58</v>
+      </c>
+      <c r="D26" s="161" t="s">
+        <v>7</v>
+      </c>
+      <c r="E26" s="135" t="s">
+        <v>28</v>
+      </c>
+      <c r="F26" s="157"/>
+      <c r="G26" s="158"/>
+    </row>
+    <row r="27" spans="2:7" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="173">
+        <v>4</v>
+      </c>
+      <c r="C27" s="179" t="s">
+        <v>56</v>
+      </c>
+      <c r="D27" s="175" t="s">
+        <v>78</v>
+      </c>
+      <c r="E27" s="123">
+        <v>192.38</v>
+      </c>
+      <c r="F27" s="157"/>
+      <c r="G27" s="158"/>
+    </row>
+    <row r="28" spans="2:7" s="105" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="170"/>
+      <c r="C28" s="180"/>
+      <c r="D28" s="172" t="s">
+        <v>81</v>
+      </c>
+      <c r="E28" s="130">
+        <f>E27</f>
+        <v>192.38</v>
+      </c>
+      <c r="F28" s="157"/>
+      <c r="G28" s="158"/>
+    </row>
+    <row r="29" spans="2:7" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="106"/>
+      <c r="C29" s="176"/>
+      <c r="D29" s="177"/>
+      <c r="E29" s="178"/>
+      <c r="F29" s="157"/>
+      <c r="G29" s="158"/>
+    </row>
+    <row r="30" spans="2:7" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="106"/>
+      <c r="C30" s="176"/>
+      <c r="D30" s="177"/>
+      <c r="E30" s="178"/>
+      <c r="F30" s="157"/>
+      <c r="G30" s="158"/>
+    </row>
+    <row r="31" spans="2:7" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="106"/>
+      <c r="C31" s="176"/>
+      <c r="D31" s="177"/>
+      <c r="E31" s="178"/>
+      <c r="F31" s="157"/>
+      <c r="G31" s="158"/>
+    </row>
+    <row r="32" spans="2:7" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="181"/>
+      <c r="C32" s="103" t="s">
+        <v>6</v>
+      </c>
+      <c r="D32" s="140" t="s">
+        <v>7</v>
+      </c>
+      <c r="E32" s="125" t="s">
+        <v>28</v>
+      </c>
+      <c r="F32" s="157"/>
+    </row>
+    <row r="33" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="181"/>
+      <c r="C33" s="103">
+        <v>1</v>
+      </c>
+      <c r="D33" s="140" t="s">
+        <v>12</v>
+      </c>
+      <c r="E33" s="125">
+        <v>340.88</v>
+      </c>
+      <c r="F33" s="157"/>
+    </row>
+    <row r="34" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="181"/>
+      <c r="C34" s="103">
+        <v>2</v>
+      </c>
+      <c r="D34" s="140" t="s">
+        <v>13</v>
+      </c>
+      <c r="E34" s="125">
+        <v>0</v>
+      </c>
+      <c r="F34" s="157"/>
+    </row>
+    <row r="35" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="181"/>
+      <c r="C35" s="103">
+        <v>3</v>
+      </c>
+      <c r="D35" s="140" t="s">
+        <v>36</v>
+      </c>
+      <c r="E35" s="125">
+        <v>340.88</v>
+      </c>
+      <c r="F35" s="157"/>
+    </row>
+    <row r="36" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B36" s="181"/>
+      <c r="C36" s="103">
+        <v>4</v>
+      </c>
+      <c r="D36" s="140" t="s">
+        <v>35</v>
+      </c>
+      <c r="E36" s="125">
+        <v>0</v>
+      </c>
+      <c r="F36" s="157"/>
+    </row>
+    <row r="37" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B37" s="181"/>
+      <c r="C37" s="103">
+        <v>5</v>
+      </c>
+      <c r="D37" s="140" t="s">
+        <v>34</v>
+      </c>
+      <c r="E37" s="125" t="s">
+        <v>26</v>
+      </c>
+      <c r="F37" s="157"/>
+      <c r="H37" s="158"/>
+    </row>
+    <row r="38" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="181"/>
+      <c r="C38" s="103">
+        <v>6</v>
+      </c>
+      <c r="D38" s="124"/>
+      <c r="E38" s="125">
+        <f>E33</f>
+        <v>340.88</v>
+      </c>
+      <c r="F38" s="157"/>
+    </row>
+    <row r="40" spans="2:8" s="152" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="41" spans="2:8" s="152" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B41" s="153"/>
+      <c r="C41" s="154"/>
+      <c r="D41" s="155"/>
+      <c r="E41" s="156"/>
+    </row>
+    <row r="42" spans="2:8" s="152" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B42" s="159" t="s">
+        <v>6</v>
+      </c>
+      <c r="C42" s="160" t="s">
+        <v>58</v>
+      </c>
+      <c r="D42" s="161" t="s">
+        <v>7</v>
+      </c>
+      <c r="E42" s="135" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="43" spans="2:8" s="152" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B43" s="162"/>
+      <c r="C43" s="163"/>
+      <c r="D43" s="164" t="s">
+        <v>78</v>
+      </c>
+      <c r="E43" s="165">
+        <f>E5+E12+E21+E27</f>
+        <v>1268.4699999999998</v>
+      </c>
+    </row>
+    <row r="44" spans="2:8" s="152" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B44" s="166"/>
+      <c r="C44" s="167"/>
+      <c r="D44" s="140" t="s">
+        <v>1</v>
+      </c>
+      <c r="E44" s="126">
+        <f>E13+E6</f>
+        <v>58.519999999999996</v>
+      </c>
+    </row>
+    <row r="45" spans="2:8" s="152" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B45" s="166"/>
+      <c r="C45" s="167"/>
+      <c r="D45" s="140" t="s">
+        <v>57</v>
+      </c>
+      <c r="E45" s="126">
+        <f>E44</f>
+        <v>58.519999999999996</v>
+      </c>
+    </row>
+    <row r="46" spans="2:8" s="152" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B46" s="166"/>
+      <c r="C46" s="167"/>
+      <c r="D46" s="168" t="s">
+        <v>11</v>
+      </c>
+      <c r="E46" s="169" t="str">
+        <f>TEXT(G46, "0.00") &amp; " п.м"</f>
+        <v>111.69 п.м</v>
+      </c>
+      <c r="G46" s="182">
+        <f>G15+G8</f>
+        <v>111.69</v>
+      </c>
+    </row>
+    <row r="47" spans="2:8" s="152" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B47" s="170"/>
+      <c r="C47" s="171"/>
+      <c r="D47" s="172" t="s">
+        <v>12</v>
+      </c>
+      <c r="E47" s="130">
+        <f>E43</f>
+        <v>1268.4699999999998</v>
+      </c>
+    </row>
+    <row r="49" spans="2:7" s="152" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="50" spans="2:7" s="152" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B50" s="153"/>
+      <c r="C50" s="154"/>
+      <c r="D50" s="155" t="s">
+        <v>9</v>
+      </c>
+      <c r="E50" s="156"/>
+    </row>
+    <row r="51" spans="2:7" s="152" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B51" s="159" t="s">
+        <v>6</v>
+      </c>
+      <c r="C51" s="160" t="s">
+        <v>58</v>
+      </c>
+      <c r="D51" s="161" t="s">
+        <v>7</v>
+      </c>
+      <c r="E51" s="135" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="52" spans="2:7" s="152" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B52" s="162">
+        <v>1</v>
+      </c>
+      <c r="C52" s="163" t="s">
+        <v>54</v>
+      </c>
+      <c r="D52" s="164" t="s">
+        <v>78</v>
+      </c>
+      <c r="E52" s="165">
+        <v>336.4</v>
+      </c>
+    </row>
+    <row r="53" spans="2:7" s="152" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B53" s="166"/>
+      <c r="C53" s="167"/>
+      <c r="D53" s="140" t="s">
+        <v>1</v>
+      </c>
+      <c r="E53" s="126">
+        <v>30.2</v>
+      </c>
+    </row>
+    <row r="54" spans="2:7" s="152" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B54" s="166"/>
+      <c r="C54" s="167"/>
+      <c r="D54" s="140" t="s">
+        <v>57</v>
+      </c>
+      <c r="E54" s="126">
+        <f>E53</f>
+        <v>30.2</v>
+      </c>
+    </row>
+    <row r="55" spans="2:7" s="152" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B55" s="166"/>
+      <c r="C55" s="167"/>
+      <c r="D55" s="168" t="s">
+        <v>11</v>
+      </c>
+      <c r="E55" s="169" t="str">
+        <f>TEXT(G55, "0.00") &amp; " п.м"</f>
+        <v>60.41 п.м</v>
+      </c>
+      <c r="G55" s="158">
+        <v>60.41</v>
+      </c>
+    </row>
+    <row r="56" spans="2:7" s="152" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B56" s="170"/>
+      <c r="C56" s="171"/>
+      <c r="D56" s="172" t="s">
+        <v>81</v>
+      </c>
+      <c r="E56" s="130">
+        <f>E52</f>
+        <v>336.4</v>
+      </c>
+      <c r="G56" s="158"/>
+    </row>
+    <row r="57" spans="2:7" s="152" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B57" s="173">
+        <v>2</v>
+      </c>
+      <c r="C57" s="174" t="s">
+        <v>77</v>
+      </c>
+      <c r="D57" s="175" t="s">
+        <v>78</v>
+      </c>
+      <c r="E57" s="123">
+        <v>543.35</v>
+      </c>
+      <c r="G57" s="158"/>
+    </row>
+    <row r="58" spans="2:7" s="152" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B58" s="166"/>
+      <c r="C58" s="167"/>
+      <c r="D58" s="140" t="s">
+        <v>1</v>
+      </c>
+      <c r="E58" s="126">
+        <v>28.32</v>
+      </c>
+      <c r="G58" s="158"/>
+    </row>
+    <row r="59" spans="2:7" s="152" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B59" s="166"/>
+      <c r="C59" s="167"/>
+      <c r="D59" s="140" t="s">
+        <v>57</v>
+      </c>
+      <c r="E59" s="126">
+        <f>E58</f>
+        <v>28.32</v>
+      </c>
+      <c r="G59" s="158"/>
+    </row>
+    <row r="60" spans="2:7" s="152" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B60" s="166"/>
+      <c r="C60" s="167"/>
+      <c r="D60" s="168" t="s">
+        <v>11</v>
+      </c>
+      <c r="E60" s="169" t="str">
+        <f>TEXT(G60, "0.00") &amp; " п.м"</f>
+        <v>51.28 п.м</v>
+      </c>
+      <c r="G60" s="158">
+        <v>51.28</v>
+      </c>
+    </row>
+    <row r="61" spans="2:7" s="152" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B61" s="170"/>
+      <c r="C61" s="171"/>
+      <c r="D61" s="172" t="s">
+        <v>81</v>
+      </c>
+      <c r="E61" s="130">
+        <f>E57</f>
+        <v>543.35</v>
+      </c>
+      <c r="G61" s="158"/>
+    </row>
+    <row r="62" spans="2:7" s="152" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="B62" s="173">
+        <v>3</v>
+      </c>
+      <c r="C62" s="179" t="s">
+        <v>79</v>
+      </c>
+      <c r="D62" s="175" t="s">
+        <v>78</v>
+      </c>
+      <c r="E62" s="123">
+        <v>196.34</v>
+      </c>
+    </row>
+    <row r="63" spans="2:7" s="152" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B63" s="170"/>
+      <c r="C63" s="180"/>
+      <c r="D63" s="172" t="s">
+        <v>81</v>
+      </c>
+      <c r="E63" s="130">
+        <f>E62</f>
+        <v>196.34</v>
+      </c>
+    </row>
+    <row r="64" spans="2:7" s="152" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B64" s="173">
+        <v>4</v>
+      </c>
+      <c r="C64" s="179" t="s">
+        <v>56</v>
+      </c>
+      <c r="D64" s="175" t="s">
+        <v>78</v>
+      </c>
+      <c r="E64" s="123">
+        <v>192.38</v>
+      </c>
+    </row>
+    <row r="65" spans="2:5" s="152" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B65" s="170"/>
+      <c r="C65" s="180"/>
+      <c r="D65" s="172" t="s">
+        <v>81</v>
+      </c>
+      <c r="E65" s="130">
+        <f>E64</f>
+        <v>192.38</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A2:G28"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="6.42578125" style="99" customWidth="1"/>
+    <col min="2" max="2" width="7.85546875" style="100" customWidth="1"/>
+    <col min="3" max="3" width="59.140625" style="99" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" style="101" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" style="109"/>
+    <col min="6" max="16384" width="9.140625" style="99"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="110"/>
+      <c r="B3" s="111"/>
+      <c r="C3" s="143" t="s">
+        <v>91</v>
+      </c>
+      <c r="D3" s="112"/>
+      <c r="E3" s="113"/>
+      <c r="F3" s="114"/>
+    </row>
+    <row r="4" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="110"/>
+      <c r="B4" s="115" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="116" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="117" t="s">
+        <v>68</v>
+      </c>
+      <c r="E4" s="118"/>
+      <c r="F4" s="114"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="119"/>
+      <c r="B5" s="120">
+        <v>1</v>
+      </c>
+      <c r="C5" s="121" t="s">
+        <v>1</v>
+      </c>
+      <c r="D5" s="122">
+        <f>G5</f>
+        <v>2606.7700000000004</v>
+      </c>
+      <c r="E5" s="123" t="s">
+        <v>69</v>
+      </c>
+      <c r="F5" s="114"/>
+      <c r="G5" s="99">
+        <f>SUM('стены штукатурка'!H1:H75)</f>
+        <v>2606.7700000000004</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="B6" s="107">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C6" s="124" t="s">
+        <v>73</v>
+      </c>
+      <c r="D6" s="125">
+        <v>991.77</v>
+      </c>
+      <c r="E6" s="126" t="s">
+        <v>69</v>
+      </c>
+      <c r="F6" s="114"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B7" s="107" t="s">
+        <v>61</v>
+      </c>
+      <c r="C7" s="127" t="s">
+        <v>60</v>
+      </c>
+      <c r="D7" s="125">
+        <f>D6*1.3</f>
+        <v>1289.3009999999999</v>
+      </c>
+      <c r="E7" s="126" t="s">
+        <v>72</v>
+      </c>
+      <c r="F7" s="114"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B8" s="107" t="s">
+        <v>62</v>
+      </c>
+      <c r="C8" s="127" t="s">
+        <v>75</v>
+      </c>
+      <c r="D8" s="125">
+        <f>D6*1.1</f>
+        <v>1090.9470000000001</v>
+      </c>
+      <c r="E8" s="126" t="s">
+        <v>69</v>
+      </c>
+      <c r="F8" s="114"/>
+    </row>
+    <row r="9" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="108" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="128" t="s">
+        <v>71</v>
+      </c>
+      <c r="D9" s="129">
+        <f>D6*0.25</f>
+        <v>247.9425</v>
+      </c>
+      <c r="E9" s="130" t="s">
+        <v>72</v>
+      </c>
+      <c r="F9" s="114"/>
+    </row>
+    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+      <c r="B10" s="120" t="s">
+        <v>64</v>
+      </c>
+      <c r="C10" s="131" t="s">
+        <v>74</v>
+      </c>
+      <c r="D10" s="122">
+        <f>D5-D6</f>
+        <v>1615.0000000000005</v>
+      </c>
+      <c r="E10" s="123" t="s">
+        <v>69</v>
+      </c>
+      <c r="F10" s="114"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B11" s="107" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" s="127" t="s">
+        <v>76</v>
+      </c>
+      <c r="D11" s="125">
+        <f>D10*1.3</f>
+        <v>2099.5000000000005</v>
+      </c>
+      <c r="E11" s="126" t="s">
+        <v>72</v>
+      </c>
+      <c r="F11" s="114"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B12" s="107" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" s="127" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12" s="125">
+        <f>D10</f>
+        <v>1615.0000000000005</v>
+      </c>
+      <c r="E12" s="126" t="s">
+        <v>69</v>
+      </c>
+      <c r="F12" s="114"/>
+    </row>
+    <row r="13" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="108" t="s">
+        <v>67</v>
+      </c>
+      <c r="C13" s="128" t="s">
+        <v>60</v>
+      </c>
+      <c r="D13" s="129">
+        <f>D10*0.25</f>
+        <v>403.75000000000011</v>
+      </c>
+      <c r="E13" s="130" t="s">
+        <v>72</v>
+      </c>
+      <c r="F13" s="114"/>
+    </row>
+    <row r="14" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="132">
+        <v>2</v>
+      </c>
+      <c r="C14" s="133" t="s">
+        <v>57</v>
+      </c>
+      <c r="D14" s="134">
+        <f>D12+D8</f>
+        <v>2705.9470000000006</v>
+      </c>
+      <c r="E14" s="135" t="s">
+        <v>69</v>
+      </c>
+      <c r="F14" s="114"/>
+    </row>
+    <row r="15" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="136">
+        <v>3</v>
+      </c>
+      <c r="C15" s="137" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="138">
+        <v>717.45</v>
+      </c>
+      <c r="E15" s="139" t="s">
+        <v>70</v>
+      </c>
+      <c r="F15" s="114"/>
+    </row>
+    <row r="17" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" s="105"/>
+      <c r="B18" s="142"/>
+      <c r="C18" s="143" t="s">
+        <v>91</v>
+      </c>
+      <c r="D18" s="143"/>
+      <c r="E18" s="144"/>
+    </row>
+    <row r="19" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="105"/>
+      <c r="B19" s="115" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" s="148" t="s">
+        <v>7</v>
+      </c>
+      <c r="D19" s="117" t="s">
+        <v>68</v>
+      </c>
+      <c r="E19" s="151"/>
+    </row>
+    <row r="20" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="105"/>
+      <c r="B20" s="136" t="s">
+        <v>82</v>
+      </c>
+      <c r="C20" s="149" t="s">
+        <v>78</v>
+      </c>
+      <c r="D20" s="150">
+        <v>1268.4699999999998</v>
+      </c>
+      <c r="E20" s="139" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" s="105"/>
+      <c r="B21" s="120" t="s">
+        <v>83</v>
+      </c>
+      <c r="C21" s="145" t="s">
+        <v>1</v>
+      </c>
+      <c r="D21" s="146">
+        <v>58.519999999999996</v>
+      </c>
+      <c r="E21" s="123" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="105"/>
+      <c r="B22" s="107" t="s">
+        <v>84</v>
+      </c>
+      <c r="C22" s="140" t="s">
+        <v>76</v>
+      </c>
+      <c r="D22" s="103">
+        <f>D21*0.25</f>
+        <v>14.629999999999999</v>
+      </c>
+      <c r="E22" s="126" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="105"/>
+      <c r="B23" s="107" t="s">
+        <v>85</v>
+      </c>
+      <c r="C23" s="102" t="s">
+        <v>60</v>
+      </c>
+      <c r="D23" s="125">
+        <f>D21*0.15</f>
+        <v>8.7779999999999987</v>
+      </c>
+      <c r="E23" s="126" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" s="105"/>
+      <c r="B24" s="107" t="s">
+        <v>86</v>
+      </c>
+      <c r="C24" s="102" t="s">
+        <v>57</v>
+      </c>
+      <c r="D24" s="103">
+        <v>58.519999999999996</v>
+      </c>
+      <c r="E24" s="126" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="105"/>
+      <c r="B25" s="108" t="s">
+        <v>87</v>
+      </c>
+      <c r="C25" s="104" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" s="141">
+        <v>111.69</v>
+      </c>
+      <c r="E25" s="147" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="105"/>
+      <c r="B26" s="120" t="s">
+        <v>88</v>
+      </c>
+      <c r="C26" s="145" t="s">
+        <v>81</v>
+      </c>
+      <c r="D26" s="146">
+        <v>1268.4699999999998</v>
+      </c>
+      <c r="E26" s="123" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="105"/>
+      <c r="B27" s="107" t="s">
+        <v>89</v>
+      </c>
+      <c r="C27" s="102" t="s">
+        <v>80</v>
+      </c>
+      <c r="D27" s="125">
+        <f>D26*4.5</f>
+        <v>5708.1149999999989</v>
+      </c>
+      <c r="E27" s="126" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="108" t="s">
+        <v>90</v>
+      </c>
+      <c r="C28" s="104" t="s">
+        <v>92</v>
+      </c>
+      <c r="D28" s="129">
+        <f>D26*0.15</f>
+        <v>190.27049999999997</v>
+      </c>
+      <c r="E28" s="130" t="s">
+        <v>72</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Update as_building drawing v1.18 spartak
</commit_message>
<xml_diff>
--- a/vor_lublino.xlsx
+++ b/vor_lublino.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="23265" yWindow="5565" windowWidth="5535" windowHeight="6105" firstSheet="2" activeTab="5"/>
+    <workbookView xWindow="23265" yWindow="5565" windowWidth="5535" windowHeight="6105" firstSheet="2" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Пример" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="98">
   <si>
     <t>Штукатурка цементным составом толщиной 16‐20 мм</t>
   </si>
@@ -298,6 +298,21 @@
   </si>
   <si>
     <t>Грунт универсальный ЛАСТИМИН</t>
+  </si>
+  <si>
+    <t>Ведомость работ и используемых материалов</t>
+  </si>
+  <si>
+    <t>1.038</t>
+  </si>
+  <si>
+    <t>1.037</t>
+  </si>
+  <si>
+    <t>1.035</t>
+  </si>
+  <si>
+    <t>1.034</t>
   </si>
 </sst>
 </file>
@@ -2912,7 +2927,7 @@
       <c r="A3" s="51"/>
       <c r="B3" s="90"/>
       <c r="C3" s="91" t="s">
-        <v>9</v>
+        <v>93</v>
       </c>
       <c r="D3" s="92"/>
       <c r="E3" s="93"/>
@@ -4105,7 +4120,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:H65"/>
+  <dimension ref="B2:H78"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="152"/>
@@ -4117,7 +4132,7 @@
     <col min="7" max="16384" width="9.140625" style="152"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" s="152" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="2:8" s="105" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="153"/>
       <c r="C3" s="154"/>
@@ -4573,14 +4588,14 @@
       </c>
       <c r="F38" s="157"/>
     </row>
-    <row r="40" spans="2:8" s="152" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="41" spans="2:8" s="152" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="41" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B41" s="153"/>
       <c r="C41" s="154"/>
       <c r="D41" s="155"/>
       <c r="E41" s="156"/>
     </row>
-    <row r="42" spans="2:8" s="152" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B42" s="159" t="s">
         <v>6</v>
       </c>
@@ -4594,7 +4609,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="43" spans="2:8" s="152" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B43" s="162"/>
       <c r="C43" s="163"/>
       <c r="D43" s="164" t="s">
@@ -4605,7 +4620,7 @@
         <v>1268.4699999999998</v>
       </c>
     </row>
-    <row r="44" spans="2:8" s="152" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B44" s="166"/>
       <c r="C44" s="167"/>
       <c r="D44" s="140" t="s">
@@ -4616,7 +4631,7 @@
         <v>58.519999999999996</v>
       </c>
     </row>
-    <row r="45" spans="2:8" s="152" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B45" s="166"/>
       <c r="C45" s="167"/>
       <c r="D45" s="140" t="s">
@@ -4627,7 +4642,7 @@
         <v>58.519999999999996</v>
       </c>
     </row>
-    <row r="46" spans="2:8" s="152" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B46" s="166"/>
       <c r="C46" s="167"/>
       <c r="D46" s="168" t="s">
@@ -4642,7 +4657,7 @@
         <v>111.69</v>
       </c>
     </row>
-    <row r="47" spans="2:8" s="152" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B47" s="170"/>
       <c r="C47" s="171"/>
       <c r="D47" s="172" t="s">
@@ -4653,8 +4668,8 @@
         <v>1268.4699999999998</v>
       </c>
     </row>
-    <row r="49" spans="2:7" s="152" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="50" spans="2:7" s="152" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="50" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B50" s="153"/>
       <c r="C50" s="154"/>
       <c r="D50" s="155" t="s">
@@ -4662,7 +4677,7 @@
       </c>
       <c r="E50" s="156"/>
     </row>
-    <row r="51" spans="2:7" s="152" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B51" s="159" t="s">
         <v>6</v>
       </c>
@@ -4676,7 +4691,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="52" spans="2:7" s="152" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B52" s="162">
         <v>1</v>
       </c>
@@ -4690,7 +4705,7 @@
         <v>336.4</v>
       </c>
     </row>
-    <row r="53" spans="2:7" s="152" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B53" s="166"/>
       <c r="C53" s="167"/>
       <c r="D53" s="140" t="s">
@@ -4700,7 +4715,7 @@
         <v>30.2</v>
       </c>
     </row>
-    <row r="54" spans="2:7" s="152" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B54" s="166"/>
       <c r="C54" s="167"/>
       <c r="D54" s="140" t="s">
@@ -4711,7 +4726,7 @@
         <v>30.2</v>
       </c>
     </row>
-    <row r="55" spans="2:7" s="152" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B55" s="166"/>
       <c r="C55" s="167"/>
       <c r="D55" s="168" t="s">
@@ -4725,7 +4740,7 @@
         <v>60.41</v>
       </c>
     </row>
-    <row r="56" spans="2:7" s="152" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B56" s="170"/>
       <c r="C56" s="171"/>
       <c r="D56" s="172" t="s">
@@ -4737,7 +4752,7 @@
       </c>
       <c r="G56" s="158"/>
     </row>
-    <row r="57" spans="2:7" s="152" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B57" s="173">
         <v>2</v>
       </c>
@@ -4752,7 +4767,7 @@
       </c>
       <c r="G57" s="158"/>
     </row>
-    <row r="58" spans="2:7" s="152" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B58" s="166"/>
       <c r="C58" s="167"/>
       <c r="D58" s="140" t="s">
@@ -4763,7 +4778,7 @@
       </c>
       <c r="G58" s="158"/>
     </row>
-    <row r="59" spans="2:7" s="152" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B59" s="166"/>
       <c r="C59" s="167"/>
       <c r="D59" s="140" t="s">
@@ -4775,7 +4790,7 @@
       </c>
       <c r="G59" s="158"/>
     </row>
-    <row r="60" spans="2:7" s="152" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B60" s="166"/>
       <c r="C60" s="167"/>
       <c r="D60" s="168" t="s">
@@ -4789,7 +4804,7 @@
         <v>51.28</v>
       </c>
     </row>
-    <row r="61" spans="2:7" s="152" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B61" s="170"/>
       <c r="C61" s="171"/>
       <c r="D61" s="172" t="s">
@@ -4801,21 +4816,25 @@
       </c>
       <c r="G61" s="158"/>
     </row>
-    <row r="62" spans="2:7" s="152" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B62" s="173">
         <v>3</v>
       </c>
       <c r="C62" s="179" t="s">
-        <v>79</v>
+        <v>47</v>
       </c>
       <c r="D62" s="175" t="s">
         <v>78</v>
       </c>
       <c r="E62" s="123">
-        <v>196.34</v>
-      </c>
-    </row>
-    <row r="63" spans="2:7" s="152" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>143.85999999999999</v>
+      </c>
+      <c r="F62" s="182">
+        <f>E62</f>
+        <v>143.85999999999999</v>
+      </c>
+    </row>
+    <row r="63" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B63" s="170"/>
       <c r="C63" s="180"/>
       <c r="D63" s="172" t="s">
@@ -4823,24 +4842,28 @@
       </c>
       <c r="E63" s="130">
         <f>E62</f>
-        <v>196.34</v>
-      </c>
-    </row>
-    <row r="64" spans="2:7" s="152" customFormat="1" x14ac:dyDescent="0.25">
+        <v>143.85999999999999</v>
+      </c>
+    </row>
+    <row r="64" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B64" s="173">
         <v>4</v>
       </c>
       <c r="C64" s="179" t="s">
-        <v>56</v>
+        <v>94</v>
       </c>
       <c r="D64" s="175" t="s">
         <v>78</v>
       </c>
       <c r="E64" s="123">
-        <v>192.38</v>
-      </c>
-    </row>
-    <row r="65" spans="2:5" s="152" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>5.24</v>
+      </c>
+      <c r="F64" s="182">
+        <f>E64</f>
+        <v>5.24</v>
+      </c>
+    </row>
+    <row r="65" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B65" s="170"/>
       <c r="C65" s="180"/>
       <c r="D65" s="172" t="s">
@@ -4848,7 +4871,160 @@
       </c>
       <c r="E65" s="130">
         <f>E64</f>
+        <v>5.24</v>
+      </c>
+    </row>
+    <row r="66" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B66" s="173">
+        <v>5</v>
+      </c>
+      <c r="C66" s="179" t="s">
+        <v>95</v>
+      </c>
+      <c r="D66" s="175" t="s">
+        <v>78</v>
+      </c>
+      <c r="E66" s="123">
+        <v>12.32</v>
+      </c>
+      <c r="F66" s="182">
+        <f>E66</f>
+        <v>12.32</v>
+      </c>
+    </row>
+    <row r="67" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B67" s="170"/>
+      <c r="C67" s="180"/>
+      <c r="D67" s="172" t="s">
+        <v>81</v>
+      </c>
+      <c r="E67" s="130">
+        <f>E66</f>
+        <v>12.32</v>
+      </c>
+    </row>
+    <row r="68" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B68" s="173">
+        <v>6</v>
+      </c>
+      <c r="C68" s="179" t="s">
+        <v>53</v>
+      </c>
+      <c r="D68" s="175" t="s">
+        <v>78</v>
+      </c>
+      <c r="E68" s="123">
+        <v>5.67</v>
+      </c>
+      <c r="F68" s="182">
+        <f>E68</f>
+        <v>5.67</v>
+      </c>
+    </row>
+    <row r="69" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B69" s="170"/>
+      <c r="C69" s="180"/>
+      <c r="D69" s="172" t="s">
+        <v>81</v>
+      </c>
+      <c r="E69" s="130">
+        <f>E68</f>
+        <v>5.67</v>
+      </c>
+    </row>
+    <row r="70" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B70" s="173">
+        <v>7</v>
+      </c>
+      <c r="C70" s="179" t="s">
+        <v>96</v>
+      </c>
+      <c r="D70" s="175" t="s">
+        <v>78</v>
+      </c>
+      <c r="E70" s="123">
+        <v>12.01</v>
+      </c>
+      <c r="F70" s="182">
+        <f>E70</f>
+        <v>12.01</v>
+      </c>
+    </row>
+    <row r="71" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B71" s="170"/>
+      <c r="C71" s="180"/>
+      <c r="D71" s="172" t="s">
+        <v>81</v>
+      </c>
+      <c r="E71" s="130">
+        <f>E70</f>
+        <v>12.01</v>
+      </c>
+    </row>
+    <row r="72" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B72" s="173">
+        <v>8</v>
+      </c>
+      <c r="C72" s="179" t="s">
+        <v>97</v>
+      </c>
+      <c r="D72" s="175" t="s">
+        <v>78</v>
+      </c>
+      <c r="E72" s="123">
+        <v>17.239999999999998</v>
+      </c>
+      <c r="F72" s="182">
+        <f>E72</f>
+        <v>17.239999999999998</v>
+      </c>
+    </row>
+    <row r="73" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B73" s="170"/>
+      <c r="C73" s="180"/>
+      <c r="D73" s="172" t="s">
+        <v>81</v>
+      </c>
+      <c r="E73" s="130">
+        <f>E72</f>
+        <v>17.239999999999998</v>
+      </c>
+    </row>
+    <row r="74" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B74" s="173">
+        <v>9</v>
+      </c>
+      <c r="C74" s="179" t="s">
+        <v>56</v>
+      </c>
+      <c r="D74" s="175" t="s">
+        <v>78</v>
+      </c>
+      <c r="E74" s="123">
         <v>192.38</v>
+      </c>
+    </row>
+    <row r="75" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B75" s="170"/>
+      <c r="C75" s="180"/>
+      <c r="D75" s="172" t="s">
+        <v>81</v>
+      </c>
+      <c r="E75" s="130">
+        <f>E74</f>
+        <v>192.38</v>
+      </c>
+    </row>
+    <row r="76" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="F76" s="182">
+        <f>SUM(F62:F73)</f>
+        <v>196.33999999999997</v>
+      </c>
+    </row>
+    <row r="78" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="F78" s="182">
+        <f>F76-196.34</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -5059,7 +5235,7 @@
       </c>
       <c r="F14" s="114"/>
     </row>
-    <row r="15" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B15" s="136">
         <v>3</v>
       </c>
@@ -5079,7 +5255,7 @@
       <c r="A18" s="105"/>
       <c r="B18" s="142"/>
       <c r="C18" s="143" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D18" s="143"/>
       <c r="E18" s="144"/>

</xml_diff>

<commit_message>
Update as_building drawing v1.19
</commit_message>
<xml_diff>
--- a/vor_lublino.xlsx
+++ b/vor_lublino.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="23265" yWindow="5565" windowWidth="5535" windowHeight="6105" firstSheet="2" activeTab="4"/>
+    <workbookView xWindow="23265" yWindow="5565" windowWidth="5535" windowHeight="6105" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Пример" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="101">
   <si>
     <t>Штукатурка цементным составом толщиной 16‐20 мм</t>
   </si>
@@ -279,27 +279,9 @@
     <t>2.2</t>
   </si>
   <si>
-    <t>2.3</t>
-  </si>
-  <si>
-    <t>2.4</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>3.1</t>
-  </si>
-  <si>
-    <t>3.2</t>
-  </si>
-  <si>
     <t>Ведомость используемых материалов</t>
   </si>
   <si>
-    <t>Грунт универсальный ЛАСТИМИН</t>
-  </si>
-  <si>
     <t>Ведомость работ и используемых материалов</t>
   </si>
   <si>
@@ -313,13 +295,43 @@
   </si>
   <si>
     <t>1.034</t>
+  </si>
+  <si>
+    <t>Ед. изм.</t>
+  </si>
+  <si>
+    <t>Профиль маячковый</t>
+  </si>
+  <si>
+    <t>1.1.4</t>
+  </si>
+  <si>
+    <t>1.2.4</t>
+  </si>
+  <si>
+    <t>Коэф. расхода</t>
+  </si>
+  <si>
+    <t>Штукатурка стен цементным, цементно-песчаным раствором с предварительной огрунтовкой от 21 до 40 мм</t>
+  </si>
+  <si>
+    <t>Сетка штукатурная_/пластиковая/10*10</t>
+  </si>
+  <si>
+    <t>Грунтовка универсальный ЛАСТИМИН_ / LP-51 А</t>
+  </si>
+  <si>
+    <t>Грунтовка БЕТОН-КОНТАКТ_/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="9" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+  </numFmts>
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -386,6 +398,11 @@
       <family val="2"/>
       <charset val="204"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -395,7 +412,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="40">
+  <borders count="36">
     <border>
       <left/>
       <right/>
@@ -518,19 +535,6 @@
       <right/>
       <top/>
       <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -696,69 +700,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -932,11 +873,38 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="183">
+  <cellXfs count="174">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1054,54 +1022,42 @@
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1111,97 +1067,43 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1210,11 +1112,8 @@
     <xf numFmtId="2" fontId="1" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1223,36 +1122,33 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1261,11 +1157,8 @@
     <xf numFmtId="2" fontId="6" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1274,7 +1167,7 @@
     <xf numFmtId="2" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1283,7 +1176,7 @@
     <xf numFmtId="2" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1295,105 +1188,81 @@
     <xf numFmtId="2" fontId="5" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1402,10 +1271,10 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1414,7 +1283,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="8" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1442,9 +1311,92 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="4"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="4"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
+    <cellStyle name="Обычный 2" xfId="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1901,7 +1853,7 @@
   <cols>
     <col min="1" max="1" width="9.140625" style="13"/>
     <col min="2" max="2" width="9.140625" style="21"/>
-    <col min="3" max="3" width="13.7109375" style="59" customWidth="1"/>
+    <col min="3" max="3" width="13.7109375" style="56" customWidth="1"/>
     <col min="4" max="4" width="45.85546875" style="21" customWidth="1"/>
     <col min="5" max="5" width="12.7109375" style="12" customWidth="1"/>
     <col min="6" max="6" width="10.7109375" style="12" customWidth="1"/>
@@ -1920,40 +1872,40 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="51"/>
-      <c r="B3" s="56"/>
+      <c r="B3" s="53"/>
       <c r="C3" s="60"/>
-      <c r="D3" s="57" t="s">
+      <c r="D3" s="146" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="58"/>
+      <c r="E3" s="54"/>
     </row>
     <row r="4" spans="1:8" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="51"/>
-      <c r="B4" s="64" t="s">
+      <c r="B4" s="55" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="65" t="s">
+      <c r="C4" s="147" t="s">
         <v>58</v>
       </c>
-      <c r="D4" s="66" t="s">
+      <c r="D4" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="67" t="s">
+      <c r="E4" s="46" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="51"/>
-      <c r="B5" s="53">
-        <v>1</v>
-      </c>
-      <c r="C5" s="68" t="s">
+      <c r="B5" s="61">
+        <v>1</v>
+      </c>
+      <c r="C5" s="59" t="s">
         <v>56</v>
       </c>
-      <c r="D5" s="69" t="s">
-        <v>1</v>
-      </c>
-      <c r="E5" s="54">
+      <c r="D5" s="38" t="s">
+        <v>1</v>
+      </c>
+      <c r="E5" s="47">
         <v>284.86</v>
       </c>
       <c r="H5" s="37">
@@ -1961,10 +1913,10 @@
         <v>284.86</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" s="51"/>
       <c r="B6" s="43"/>
-      <c r="C6" s="61"/>
+      <c r="C6" s="57"/>
       <c r="D6" s="15" t="s">
         <v>57</v>
       </c>
@@ -1973,10 +1925,10 @@
         <v>284.86</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" s="51"/>
       <c r="B7" s="43"/>
-      <c r="C7" s="61"/>
+      <c r="C7" s="57"/>
       <c r="D7" s="17" t="s">
         <v>11</v>
       </c>
@@ -1988,27 +1940,27 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:8" s="42" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" s="42" customFormat="1" ht="13.5" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="51"/>
-      <c r="B8" s="64"/>
-      <c r="C8" s="70"/>
-      <c r="D8" s="66"/>
-      <c r="E8" s="67"/>
+      <c r="B8" s="43"/>
+      <c r="C8" s="57"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="44"/>
       <c r="F8" s="40"/>
       <c r="G8" s="41"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="51"/>
-      <c r="B9" s="53">
+      <c r="B9" s="43">
         <v>2</v>
       </c>
-      <c r="C9" s="68">
+      <c r="C9" s="57">
         <v>1.0269999999999999</v>
       </c>
-      <c r="D9" s="69" t="s">
-        <v>1</v>
-      </c>
-      <c r="E9" s="54">
+      <c r="D9" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="E9" s="44">
         <v>110.55</v>
       </c>
       <c r="H9" s="37">
@@ -2016,10 +1968,10 @@
         <v>110.55</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" s="51"/>
       <c r="B10" s="43"/>
-      <c r="C10" s="61"/>
+      <c r="C10" s="57"/>
       <c r="D10" s="15" t="s">
         <v>57</v>
       </c>
@@ -2028,10 +1980,10 @@
         <v>110.55</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" s="51"/>
       <c r="B11" s="43"/>
-      <c r="C11" s="61"/>
+      <c r="C11" s="57"/>
       <c r="D11" s="17" t="s">
         <v>11</v>
       </c>
@@ -2043,27 +1995,27 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:8" s="42" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" s="42" customFormat="1" ht="13.5" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="51"/>
-      <c r="B12" s="55"/>
-      <c r="C12" s="62"/>
-      <c r="D12" s="39"/>
-      <c r="E12" s="46"/>
+      <c r="B12" s="43"/>
+      <c r="C12" s="57"/>
+      <c r="D12" s="15"/>
+      <c r="E12" s="44"/>
       <c r="F12" s="40"/>
       <c r="G12" s="41"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" s="51"/>
-      <c r="B13" s="71">
+      <c r="B13" s="43">
         <v>3</v>
       </c>
-      <c r="C13" s="63" t="s">
+      <c r="C13" s="57" t="s">
         <v>59</v>
       </c>
-      <c r="D13" s="38" t="s">
-        <v>1</v>
-      </c>
-      <c r="E13" s="47">
+      <c r="D13" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="E13" s="44">
         <v>103.27</v>
       </c>
       <c r="H13" s="37">
@@ -2071,10 +2023,10 @@
         <v>103.27</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" s="51"/>
       <c r="B14" s="43"/>
-      <c r="C14" s="61"/>
+      <c r="C14" s="57"/>
       <c r="D14" s="15" t="s">
         <v>57</v>
       </c>
@@ -2083,10 +2035,10 @@
         <v>103.27</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" s="51"/>
       <c r="B15" s="43"/>
-      <c r="C15" s="61"/>
+      <c r="C15" s="57"/>
       <c r="D15" s="17" t="s">
         <v>11</v>
       </c>
@@ -2095,27 +2047,27 @@
         <v>0.00 п.м</v>
       </c>
     </row>
-    <row r="16" spans="1:8" s="42" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" s="42" customFormat="1" ht="13.5" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A16" s="51"/>
-      <c r="B16" s="64"/>
-      <c r="C16" s="70"/>
-      <c r="D16" s="66"/>
-      <c r="E16" s="67"/>
+      <c r="B16" s="43"/>
+      <c r="C16" s="57"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="44"/>
       <c r="F16" s="40"/>
       <c r="G16" s="41"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="51"/>
-      <c r="B17" s="53">
+      <c r="B17" s="43">
         <v>4</v>
       </c>
-      <c r="C17" s="68">
+      <c r="C17" s="57">
         <v>1.0289999999999999</v>
       </c>
-      <c r="D17" s="69" t="s">
-        <v>1</v>
-      </c>
-      <c r="E17" s="54">
+      <c r="D17" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="E17" s="44">
         <v>92.42</v>
       </c>
       <c r="H17" s="37">
@@ -2123,10 +2075,10 @@
         <v>92.42</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" s="51"/>
       <c r="B18" s="43"/>
-      <c r="C18" s="61"/>
+      <c r="C18" s="57"/>
       <c r="D18" s="15" t="s">
         <v>57</v>
       </c>
@@ -2135,10 +2087,10 @@
         <v>92.42</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" s="51"/>
       <c r="B19" s="43"/>
-      <c r="C19" s="61"/>
+      <c r="C19" s="57"/>
       <c r="D19" s="17" t="s">
         <v>11</v>
       </c>
@@ -2147,27 +2099,27 @@
         <v>0.00 п.м</v>
       </c>
     </row>
-    <row r="20" spans="1:8" s="42" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" s="42" customFormat="1" ht="13.5" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A20" s="51"/>
-      <c r="B20" s="55"/>
-      <c r="C20" s="62"/>
-      <c r="D20" s="39"/>
-      <c r="E20" s="46"/>
+      <c r="B20" s="43"/>
+      <c r="C20" s="57"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="44"/>
       <c r="F20" s="40"/>
       <c r="G20" s="41"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A21" s="51"/>
-      <c r="B21" s="71">
+      <c r="B21" s="43">
         <v>5</v>
       </c>
-      <c r="C21" s="63" t="s">
+      <c r="C21" s="57" t="s">
         <v>50</v>
       </c>
-      <c r="D21" s="38" t="s">
-        <v>1</v>
-      </c>
-      <c r="E21" s="47">
+      <c r="D21" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="E21" s="44">
         <v>94.91</v>
       </c>
       <c r="H21" s="37">
@@ -2175,10 +2127,10 @@
         <v>94.91</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" s="51"/>
       <c r="B22" s="43"/>
-      <c r="C22" s="61"/>
+      <c r="C22" s="57"/>
       <c r="D22" s="15" t="s">
         <v>57</v>
       </c>
@@ -2187,10 +2139,10 @@
         <v>94.91</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" s="51"/>
       <c r="B23" s="43"/>
-      <c r="C23" s="61"/>
+      <c r="C23" s="57"/>
       <c r="D23" s="17" t="s">
         <v>11</v>
       </c>
@@ -2198,27 +2150,27 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="1:8" s="42" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" s="42" customFormat="1" ht="13.5" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A24" s="51"/>
-      <c r="B24" s="64"/>
-      <c r="C24" s="70"/>
-      <c r="D24" s="66"/>
-      <c r="E24" s="67"/>
+      <c r="B24" s="43"/>
+      <c r="C24" s="57"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="44"/>
       <c r="F24" s="40"/>
       <c r="G24" s="41"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A25" s="51"/>
-      <c r="B25" s="53">
+      <c r="B25" s="43">
         <v>6</v>
       </c>
-      <c r="C25" s="68">
+      <c r="C25" s="57">
         <v>1.0309999999999999</v>
       </c>
-      <c r="D25" s="69" t="s">
-        <v>1</v>
-      </c>
-      <c r="E25" s="54">
+      <c r="D25" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="E25" s="44">
         <v>90.2</v>
       </c>
       <c r="H25" s="37">
@@ -2226,10 +2178,10 @@
         <v>90.2</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" s="51"/>
       <c r="B26" s="43"/>
-      <c r="C26" s="61"/>
+      <c r="C26" s="57"/>
       <c r="D26" s="15" t="s">
         <v>57</v>
       </c>
@@ -2238,10 +2190,10 @@
         <v>90.2</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" s="51"/>
       <c r="B27" s="43"/>
-      <c r="C27" s="61"/>
+      <c r="C27" s="57"/>
       <c r="D27" s="17" t="s">
         <v>11</v>
       </c>
@@ -2250,27 +2202,27 @@
         <v>0.00 п.м</v>
       </c>
     </row>
-    <row r="28" spans="1:8" s="42" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" s="42" customFormat="1" ht="13.5" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A28" s="51"/>
-      <c r="B28" s="55"/>
-      <c r="C28" s="62"/>
-      <c r="D28" s="39"/>
-      <c r="E28" s="46"/>
+      <c r="B28" s="43"/>
+      <c r="C28" s="57"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="44"/>
       <c r="F28" s="40"/>
       <c r="G28" s="41"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A29" s="51"/>
-      <c r="B29" s="71">
+      <c r="B29" s="43">
         <v>7</v>
       </c>
-      <c r="C29" s="63" t="s">
+      <c r="C29" s="57" t="s">
         <v>51</v>
       </c>
-      <c r="D29" s="38" t="s">
-        <v>1</v>
-      </c>
-      <c r="E29" s="47">
+      <c r="D29" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="E29" s="44">
         <v>87.76</v>
       </c>
       <c r="H29" s="37">
@@ -2278,10 +2230,10 @@
         <v>87.76</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" s="51"/>
       <c r="B30" s="43"/>
-      <c r="C30" s="61"/>
+      <c r="C30" s="57"/>
       <c r="D30" s="15" t="s">
         <v>57</v>
       </c>
@@ -2290,10 +2242,10 @@
         <v>87.76</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" s="51"/>
       <c r="B31" s="43"/>
-      <c r="C31" s="61"/>
+      <c r="C31" s="57"/>
       <c r="D31" s="17" t="s">
         <v>11</v>
       </c>
@@ -2304,27 +2256,27 @@
         <v>4</v>
       </c>
     </row>
-    <row r="32" spans="1:8" s="42" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" s="42" customFormat="1" ht="13.5" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A32" s="51"/>
-      <c r="B32" s="64"/>
-      <c r="C32" s="70"/>
-      <c r="D32" s="66"/>
-      <c r="E32" s="67"/>
+      <c r="B32" s="43"/>
+      <c r="C32" s="57"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="44"/>
       <c r="F32" s="40"/>
       <c r="G32" s="41"/>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A33" s="51"/>
-      <c r="B33" s="53">
+      <c r="B33" s="43">
         <v>8</v>
       </c>
-      <c r="C33" s="68" t="s">
+      <c r="C33" s="57" t="s">
         <v>52</v>
       </c>
-      <c r="D33" s="69" t="s">
-        <v>1</v>
-      </c>
-      <c r="E33" s="54">
+      <c r="D33" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="E33" s="44">
         <v>142.44</v>
       </c>
       <c r="H33" s="37">
@@ -2332,10 +2284,10 @@
         <v>142.44</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34" s="51"/>
       <c r="B34" s="43"/>
-      <c r="C34" s="61"/>
+      <c r="C34" s="57"/>
       <c r="D34" s="15" t="s">
         <v>57</v>
       </c>
@@ -2344,10 +2296,10 @@
         <v>142.44</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" s="51"/>
       <c r="B35" s="43"/>
-      <c r="C35" s="61"/>
+      <c r="C35" s="57"/>
       <c r="D35" s="17" t="s">
         <v>11</v>
       </c>
@@ -2356,27 +2308,27 @@
         <v>0.00 п.м</v>
       </c>
     </row>
-    <row r="36" spans="1:8" s="42" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" s="42" customFormat="1" ht="13.5" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A36" s="51"/>
-      <c r="B36" s="55"/>
-      <c r="C36" s="62"/>
-      <c r="D36" s="39"/>
-      <c r="E36" s="46"/>
+      <c r="B36" s="43"/>
+      <c r="C36" s="57"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="44"/>
       <c r="F36" s="40"/>
       <c r="G36" s="41"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A37" s="51"/>
-      <c r="B37" s="53">
+      <c r="B37" s="43">
         <v>9</v>
       </c>
-      <c r="C37" s="68">
+      <c r="C37" s="57">
         <v>1.034</v>
       </c>
-      <c r="D37" s="69" t="s">
-        <v>1</v>
-      </c>
-      <c r="E37" s="54">
+      <c r="D37" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="E37" s="44">
         <v>76.23</v>
       </c>
       <c r="H37" s="37">
@@ -2384,10 +2336,10 @@
         <v>76.23</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" s="51"/>
       <c r="B38" s="43"/>
-      <c r="C38" s="61"/>
+      <c r="C38" s="57"/>
       <c r="D38" s="15" t="s">
         <v>57</v>
       </c>
@@ -2396,10 +2348,10 @@
         <v>76.23</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" s="51"/>
       <c r="B39" s="43"/>
-      <c r="C39" s="61"/>
+      <c r="C39" s="57"/>
       <c r="D39" s="17" t="s">
         <v>11</v>
       </c>
@@ -2408,27 +2360,27 @@
         <v>0.00 п.м</v>
       </c>
     </row>
-    <row r="40" spans="1:8" s="42" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" s="42" customFormat="1" ht="13.5" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A40" s="51"/>
-      <c r="B40" s="55"/>
-      <c r="C40" s="62"/>
-      <c r="D40" s="39"/>
-      <c r="E40" s="46"/>
+      <c r="B40" s="43"/>
+      <c r="C40" s="57"/>
+      <c r="D40" s="15"/>
+      <c r="E40" s="44"/>
       <c r="F40" s="40"/>
       <c r="G40" s="41"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A41" s="51"/>
-      <c r="B41" s="71">
+      <c r="B41" s="43">
         <v>10</v>
       </c>
-      <c r="C41" s="63" t="s">
+      <c r="C41" s="57" t="s">
         <v>45</v>
       </c>
-      <c r="D41" s="38" t="s">
-        <v>1</v>
-      </c>
-      <c r="E41" s="47">
+      <c r="D41" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="E41" s="44">
         <v>40.76</v>
       </c>
       <c r="H41" s="37">
@@ -2436,10 +2388,10 @@
         <v>40.76</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" s="51"/>
       <c r="B42" s="43"/>
-      <c r="C42" s="61"/>
+      <c r="C42" s="57"/>
       <c r="D42" s="15" t="s">
         <v>57</v>
       </c>
@@ -2448,10 +2400,10 @@
         <v>40.76</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" s="51"/>
       <c r="B43" s="43"/>
-      <c r="C43" s="61"/>
+      <c r="C43" s="57"/>
       <c r="D43" s="17" t="s">
         <v>11</v>
       </c>
@@ -2460,27 +2412,27 @@
         <v>0.00 п.м</v>
       </c>
     </row>
-    <row r="44" spans="1:8" s="42" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" s="42" customFormat="1" ht="13.5" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A44" s="51"/>
-      <c r="B44" s="64"/>
-      <c r="C44" s="70"/>
-      <c r="D44" s="66"/>
-      <c r="E44" s="67"/>
+      <c r="B44" s="43"/>
+      <c r="C44" s="57"/>
+      <c r="D44" s="15"/>
+      <c r="E44" s="44"/>
       <c r="F44" s="40"/>
       <c r="G44" s="41"/>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A45" s="51"/>
-      <c r="B45" s="53">
+      <c r="B45" s="43">
         <v>11</v>
       </c>
-      <c r="C45" s="68" t="s">
+      <c r="C45" s="57" t="s">
         <v>53</v>
       </c>
-      <c r="D45" s="69" t="s">
-        <v>1</v>
-      </c>
-      <c r="E45" s="54">
+      <c r="D45" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="E45" s="44">
         <v>14.15</v>
       </c>
       <c r="H45" s="37">
@@ -2488,10 +2440,10 @@
         <v>14.15</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" s="51"/>
       <c r="B46" s="43"/>
-      <c r="C46" s="61"/>
+      <c r="C46" s="57"/>
       <c r="D46" s="15" t="s">
         <v>57</v>
       </c>
@@ -2500,10 +2452,10 @@
         <v>14.15</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" s="51"/>
       <c r="B47" s="43"/>
-      <c r="C47" s="61"/>
+      <c r="C47" s="57"/>
       <c r="D47" s="17" t="s">
         <v>11</v>
       </c>
@@ -2512,27 +2464,27 @@
         <v>0.00 п.м</v>
       </c>
     </row>
-    <row r="48" spans="1:8" s="42" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" s="42" customFormat="1" ht="13.5" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A48" s="51"/>
-      <c r="B48" s="55"/>
-      <c r="C48" s="62"/>
-      <c r="D48" s="39"/>
-      <c r="E48" s="46"/>
+      <c r="B48" s="43"/>
+      <c r="C48" s="57"/>
+      <c r="D48" s="15"/>
+      <c r="E48" s="44"/>
       <c r="F48" s="40"/>
       <c r="G48" s="41"/>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A49" s="51"/>
-      <c r="B49" s="71">
+      <c r="B49" s="43">
         <v>12</v>
       </c>
-      <c r="C49" s="63">
+      <c r="C49" s="57">
         <v>1.038</v>
       </c>
-      <c r="D49" s="38" t="s">
-        <v>1</v>
-      </c>
-      <c r="E49" s="47">
+      <c r="D49" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="E49" s="44">
         <v>36.69</v>
       </c>
       <c r="H49" s="37">
@@ -2540,10 +2492,10 @@
         <v>36.69</v>
       </c>
     </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50" s="51"/>
       <c r="B50" s="43"/>
-      <c r="C50" s="61"/>
+      <c r="C50" s="57"/>
       <c r="D50" s="15" t="s">
         <v>57</v>
       </c>
@@ -2552,10 +2504,10 @@
         <v>36.69</v>
       </c>
     </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51" s="51"/>
       <c r="B51" s="43"/>
-      <c r="C51" s="61"/>
+      <c r="C51" s="57"/>
       <c r="D51" s="17" t="s">
         <v>11</v>
       </c>
@@ -2564,27 +2516,27 @@
         <v>0.00 п.м</v>
       </c>
     </row>
-    <row r="52" spans="1:8" s="42" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:8" s="42" customFormat="1" ht="13.5" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A52" s="51"/>
-      <c r="B52" s="64"/>
-      <c r="C52" s="70"/>
-      <c r="D52" s="66"/>
-      <c r="E52" s="67"/>
+      <c r="B52" s="43"/>
+      <c r="C52" s="57"/>
+      <c r="D52" s="15"/>
+      <c r="E52" s="44"/>
       <c r="F52" s="40"/>
       <c r="G52" s="41"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A53" s="51"/>
-      <c r="B53" s="53">
+      <c r="B53" s="43">
         <v>13</v>
       </c>
-      <c r="C53" s="68" t="s">
+      <c r="C53" s="57" t="s">
         <v>47</v>
       </c>
-      <c r="D53" s="69" t="s">
-        <v>1</v>
-      </c>
-      <c r="E53" s="54">
+      <c r="D53" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="E53" s="44">
         <v>166.2</v>
       </c>
       <c r="H53" s="37">
@@ -2592,10 +2544,10 @@
         <v>166.2</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54" s="51"/>
       <c r="B54" s="43"/>
-      <c r="C54" s="61"/>
+      <c r="C54" s="57"/>
       <c r="D54" s="15" t="s">
         <v>57</v>
       </c>
@@ -2604,10 +2556,10 @@
         <v>166.2</v>
       </c>
     </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55" s="51"/>
       <c r="B55" s="43"/>
-      <c r="C55" s="61"/>
+      <c r="C55" s="57"/>
       <c r="D55" s="17" t="s">
         <v>11</v>
       </c>
@@ -2619,27 +2571,27 @@
         <v>4</v>
       </c>
     </row>
-    <row r="56" spans="1:8" s="42" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:8" s="42" customFormat="1" ht="13.5" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A56" s="51"/>
-      <c r="B56" s="55"/>
-      <c r="C56" s="62"/>
-      <c r="D56" s="39"/>
-      <c r="E56" s="46"/>
+      <c r="B56" s="43"/>
+      <c r="C56" s="57"/>
+      <c r="D56" s="15"/>
+      <c r="E56" s="44"/>
       <c r="F56" s="40"/>
       <c r="G56" s="41"/>
     </row>
     <row r="57" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A57" s="51"/>
-      <c r="B57" s="71">
+      <c r="B57" s="43">
         <v>14</v>
       </c>
-      <c r="C57" s="63" t="s">
+      <c r="C57" s="57" t="s">
         <v>48</v>
       </c>
-      <c r="D57" s="38" t="s">
-        <v>1</v>
-      </c>
-      <c r="E57" s="47">
+      <c r="D57" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="E57" s="44">
         <v>260.64999999999998</v>
       </c>
       <c r="H57" s="37">
@@ -2647,10 +2599,10 @@
         <v>260.64999999999998</v>
       </c>
     </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A58" s="51"/>
       <c r="B58" s="43"/>
-      <c r="C58" s="61"/>
+      <c r="C58" s="57"/>
       <c r="D58" s="15" t="s">
         <v>57</v>
       </c>
@@ -2659,10 +2611,10 @@
         <v>260.64999999999998</v>
       </c>
     </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A59" s="51"/>
       <c r="B59" s="43"/>
-      <c r="C59" s="61"/>
+      <c r="C59" s="57"/>
       <c r="D59" s="17" t="s">
         <v>11</v>
       </c>
@@ -2674,27 +2626,27 @@
         <v>103.45</v>
       </c>
     </row>
-    <row r="60" spans="1:8" s="42" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:8" s="42" customFormat="1" ht="13.5" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A60" s="51"/>
-      <c r="B60" s="64"/>
-      <c r="C60" s="70"/>
-      <c r="D60" s="66"/>
-      <c r="E60" s="67"/>
+      <c r="B60" s="43"/>
+      <c r="C60" s="57"/>
+      <c r="D60" s="15"/>
+      <c r="E60" s="44"/>
       <c r="F60" s="40"/>
       <c r="G60" s="41"/>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A61" s="51"/>
-      <c r="B61" s="53">
+      <c r="B61" s="43">
         <v>15</v>
       </c>
-      <c r="C61" s="68" t="s">
+      <c r="C61" s="57" t="s">
         <v>54</v>
       </c>
-      <c r="D61" s="69" t="s">
-        <v>1</v>
-      </c>
-      <c r="E61" s="54">
+      <c r="D61" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="E61" s="44">
         <v>372.12</v>
       </c>
       <c r="H61" s="37">
@@ -2702,10 +2654,10 @@
         <v>372.12</v>
       </c>
     </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62" s="51"/>
       <c r="B62" s="43"/>
-      <c r="C62" s="61"/>
+      <c r="C62" s="57"/>
       <c r="D62" s="15" t="s">
         <v>57</v>
       </c>
@@ -2714,10 +2666,10 @@
         <v>372.12</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A63" s="51"/>
       <c r="B63" s="43"/>
-      <c r="C63" s="61"/>
+      <c r="C63" s="57"/>
       <c r="D63" s="17" t="s">
         <v>11</v>
       </c>
@@ -2729,27 +2681,27 @@
         <v>263.5</v>
       </c>
     </row>
-    <row r="64" spans="1:8" s="42" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:8" s="42" customFormat="1" ht="13.5" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A64" s="51"/>
-      <c r="B64" s="55"/>
-      <c r="C64" s="62"/>
-      <c r="D64" s="39"/>
-      <c r="E64" s="46"/>
+      <c r="B64" s="43"/>
+      <c r="C64" s="57"/>
+      <c r="D64" s="15"/>
+      <c r="E64" s="44"/>
       <c r="F64" s="40"/>
       <c r="G64" s="41"/>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A65" s="51"/>
-      <c r="B65" s="71">
+      <c r="B65" s="43">
         <v>16</v>
       </c>
-      <c r="C65" s="63" t="s">
+      <c r="C65" s="57" t="s">
         <v>49</v>
       </c>
-      <c r="D65" s="38" t="s">
-        <v>1</v>
-      </c>
-      <c r="E65" s="47">
+      <c r="D65" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="E65" s="44">
         <v>75.8</v>
       </c>
       <c r="H65" s="37">
@@ -2757,10 +2709,10 @@
         <v>75.8</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A66" s="51"/>
       <c r="B66" s="43"/>
-      <c r="C66" s="61"/>
+      <c r="C66" s="57"/>
       <c r="D66" s="15" t="s">
         <v>57</v>
       </c>
@@ -2769,10 +2721,10 @@
         <v>75.8</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A67" s="51"/>
       <c r="B67" s="43"/>
-      <c r="C67" s="61"/>
+      <c r="C67" s="57"/>
       <c r="D67" s="17" t="s">
         <v>11</v>
       </c>
@@ -2784,27 +2736,27 @@
         <v>7.4</v>
       </c>
     </row>
-    <row r="68" spans="1:8" s="42" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:8" s="42" customFormat="1" ht="13.5" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A68" s="51"/>
-      <c r="B68" s="64"/>
-      <c r="C68" s="70"/>
-      <c r="D68" s="66"/>
-      <c r="E68" s="67"/>
+      <c r="B68" s="43"/>
+      <c r="C68" s="57"/>
+      <c r="D68" s="15"/>
+      <c r="E68" s="44"/>
       <c r="F68" s="40"/>
       <c r="G68" s="41"/>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A69" s="51"/>
-      <c r="B69" s="53">
+      <c r="B69" s="43">
         <v>17</v>
       </c>
-      <c r="C69" s="68" t="s">
+      <c r="C69" s="57" t="s">
         <v>46</v>
       </c>
-      <c r="D69" s="69" t="s">
-        <v>1</v>
-      </c>
-      <c r="E69" s="54">
+      <c r="D69" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="E69" s="44">
         <v>152.54</v>
       </c>
       <c r="H69" s="37">
@@ -2812,10 +2764,10 @@
         <v>152.54</v>
       </c>
     </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A70" s="51"/>
       <c r="B70" s="43"/>
-      <c r="C70" s="61"/>
+      <c r="C70" s="57"/>
       <c r="D70" s="15" t="s">
         <v>57</v>
       </c>
@@ -2824,10 +2776,10 @@
         <v>152.54</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A71" s="51"/>
       <c r="B71" s="43"/>
-      <c r="C71" s="61"/>
+      <c r="C71" s="57"/>
       <c r="D71" s="17" t="s">
         <v>11</v>
       </c>
@@ -2839,27 +2791,27 @@
         <v>26.2</v>
       </c>
     </row>
-    <row r="72" spans="1:8" s="42" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:8" s="42" customFormat="1" ht="13.5" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A72" s="51"/>
-      <c r="B72" s="55"/>
-      <c r="C72" s="62"/>
-      <c r="D72" s="39"/>
-      <c r="E72" s="46"/>
+      <c r="B72" s="43"/>
+      <c r="C72" s="57"/>
+      <c r="D72" s="15"/>
+      <c r="E72" s="44"/>
       <c r="F72" s="40"/>
       <c r="G72" s="41"/>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:8" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A73" s="51"/>
-      <c r="B73" s="71">
+      <c r="B73" s="55">
         <v>18</v>
       </c>
-      <c r="C73" s="63" t="s">
+      <c r="C73" s="58" t="s">
         <v>55</v>
       </c>
-      <c r="D73" s="38" t="s">
-        <v>1</v>
-      </c>
-      <c r="E73" s="47">
+      <c r="D73" s="39" t="s">
+        <v>1</v>
+      </c>
+      <c r="E73" s="46">
         <v>405.22</v>
       </c>
       <c r="H73" s="37">
@@ -2867,22 +2819,22 @@
         <v>405.22</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A74" s="51"/>
-      <c r="B74" s="43"/>
-      <c r="C74" s="61"/>
-      <c r="D74" s="15" t="s">
+      <c r="B74" s="61"/>
+      <c r="C74" s="59"/>
+      <c r="D74" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="E74" s="44">
+      <c r="E74" s="47">
         <f>E73</f>
         <v>405.22</v>
       </c>
     </row>
-    <row r="75" spans="1:8" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:8" ht="13.5" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A75" s="51"/>
       <c r="B75" s="55"/>
-      <c r="C75" s="62"/>
+      <c r="C75" s="58"/>
       <c r="D75" s="48" t="s">
         <v>11</v>
       </c>
@@ -2897,7 +2849,7 @@
     <row r="76" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A76" s="51"/>
       <c r="B76" s="18"/>
-      <c r="C76" s="63"/>
+      <c r="C76" s="59"/>
       <c r="D76" s="19"/>
       <c r="E76" s="20"/>
     </row>
@@ -2912,222 +2864,281 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:G15"/>
+  <dimension ref="A2:H16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.42578125" customWidth="1"/>
-    <col min="2" max="2" width="7.85546875" style="72" customWidth="1"/>
-    <col min="3" max="3" width="53" customWidth="1"/>
-    <col min="4" max="4" width="10.7109375" style="89" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" style="1"/>
+    <col min="2" max="2" width="7.5703125" style="62" customWidth="1"/>
+    <col min="3" max="3" width="54.85546875" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="14.5703125" style="68" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" style="68" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="1:7" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="3" spans="1:8" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A3" s="51"/>
-      <c r="B3" s="90"/>
-      <c r="C3" s="91" t="s">
+      <c r="B3" s="69"/>
+      <c r="C3" s="164" t="s">
+        <v>87</v>
+      </c>
+      <c r="D3" s="70"/>
+      <c r="E3" s="70"/>
+      <c r="F3" s="71"/>
+      <c r="G3" s="37"/>
+    </row>
+    <row r="4" spans="1:8" s="13" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="51"/>
+      <c r="B4" s="72" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="73" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="74" t="s">
+        <v>92</v>
+      </c>
+      <c r="E4" s="74" t="s">
+        <v>96</v>
+      </c>
+      <c r="F4" s="75" t="s">
+        <v>68</v>
+      </c>
+      <c r="G4" s="37"/>
+    </row>
+    <row r="5" spans="1:8" s="13" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="52"/>
+      <c r="B5" s="66">
+        <v>1</v>
+      </c>
+      <c r="C5" s="158" t="s">
+        <v>97</v>
+      </c>
+      <c r="D5" s="67" t="s">
+        <v>69</v>
+      </c>
+      <c r="E5" s="150">
+        <v>1</v>
+      </c>
+      <c r="F5" s="47">
+        <v>2606.7700000000004</v>
+      </c>
+      <c r="G5" s="37"/>
+      <c r="H5" s="163"/>
+    </row>
+    <row r="6" spans="1:8" s="13" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B6" s="63">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="C6" s="160" t="s">
+        <v>73</v>
+      </c>
+      <c r="D6" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="E6" s="151">
+        <v>1</v>
+      </c>
+      <c r="F6" s="44">
+        <v>991.77</v>
+      </c>
+      <c r="G6" s="37"/>
+    </row>
+    <row r="7" spans="1:8" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B7" s="63" t="s">
+        <v>61</v>
+      </c>
+      <c r="C7" s="161" t="s">
+        <v>60</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="E7" s="151">
+        <v>1.3</v>
+      </c>
+      <c r="F7" s="44">
+        <f>$F6*E7</f>
+        <v>1289.3009999999999</v>
+      </c>
+      <c r="G7" s="37"/>
+    </row>
+    <row r="8" spans="1:8" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B8" s="63" t="s">
+        <v>62</v>
+      </c>
+      <c r="C8" s="161" t="s">
+        <v>98</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="E8" s="151">
+        <f>E6*1.1</f>
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="F8" s="44">
+        <f>$F6*E8</f>
+        <v>1090.9470000000001</v>
+      </c>
+      <c r="G8" s="37"/>
+    </row>
+    <row r="9" spans="1:8" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B9" s="63" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="161" t="s">
         <v>93</v>
       </c>
-      <c r="D3" s="92"/>
-      <c r="E3" s="93"/>
-      <c r="F3" s="37"/>
-    </row>
-    <row r="4" spans="1:7" s="13" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="51"/>
-      <c r="B4" s="94" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="95" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="96" t="s">
-        <v>68</v>
-      </c>
-      <c r="E4" s="97"/>
-      <c r="F4" s="37"/>
-    </row>
-    <row r="5" spans="1:7" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A5" s="52"/>
-      <c r="B5" s="77">
-        <v>1</v>
-      </c>
-      <c r="C5" s="78" t="s">
-        <v>1</v>
-      </c>
-      <c r="D5" s="79">
-        <f>G5</f>
-        <v>2606.7700000000004</v>
-      </c>
-      <c r="E5" s="47" t="s">
+      <c r="D9" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="E9" s="151">
+        <v>1</v>
+      </c>
+      <c r="F9" s="44">
+        <f>$F6*E9</f>
+        <v>991.77</v>
+      </c>
+      <c r="G9" s="37"/>
+    </row>
+    <row r="10" spans="1:8" s="13" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B10" s="148" t="s">
+        <v>94</v>
+      </c>
+      <c r="C10" s="162" t="s">
+        <v>71</v>
+      </c>
+      <c r="D10" s="149" t="s">
+        <v>72</v>
+      </c>
+      <c r="E10" s="152">
+        <f>E6*0.25</f>
+        <v>0.25</v>
+      </c>
+      <c r="F10" s="44">
+        <f>$F6*E10</f>
+        <v>247.9425</v>
+      </c>
+      <c r="G10" s="37"/>
+    </row>
+    <row r="11" spans="1:8" s="13" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="155" t="s">
+        <v>64</v>
+      </c>
+      <c r="C11" s="159" t="s">
+        <v>74</v>
+      </c>
+      <c r="D11" s="156" t="s">
         <v>69</v>
       </c>
-      <c r="F5" s="37"/>
-      <c r="G5" s="13">
-        <f>SUM('стены штукатурка'!H1:H75)</f>
-        <v>2606.7700000000004</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" s="13" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="B6" s="73">
+      <c r="E11" s="157">
+        <v>1</v>
+      </c>
+      <c r="F11" s="54">
+        <v>1615.0000000000005</v>
+      </c>
+      <c r="G11" s="37"/>
+    </row>
+    <row r="12" spans="1:8" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B12" s="63" t="s">
+        <v>66</v>
+      </c>
+      <c r="C12" s="161" t="s">
+        <v>60</v>
+      </c>
+      <c r="D12" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="E12" s="151">
+        <v>1.3</v>
+      </c>
+      <c r="F12" s="44">
+        <f>$F11*E12</f>
+        <v>2099.5000000000005</v>
+      </c>
+      <c r="G12" s="37"/>
+    </row>
+    <row r="13" spans="1:8" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B13" s="63" t="s">
+        <v>65</v>
+      </c>
+      <c r="C13" s="161" t="s">
+        <v>98</v>
+      </c>
+      <c r="D13" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="E13" s="151">
+        <f>E11*1.1</f>
         <v>1.1000000000000001</v>
       </c>
-      <c r="C6" s="22" t="s">
-        <v>73</v>
-      </c>
-      <c r="D6" s="16">
-        <v>991.77</v>
-      </c>
-      <c r="E6" s="44" t="s">
-        <v>69</v>
-      </c>
-      <c r="F6" s="37"/>
-    </row>
-    <row r="7" spans="1:7" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B7" s="73" t="s">
-        <v>61</v>
-      </c>
-      <c r="C7" s="75" t="s">
-        <v>60</v>
-      </c>
-      <c r="D7" s="16">
-        <f>D6*1.3</f>
-        <v>1289.3009999999999</v>
-      </c>
-      <c r="E7" s="44" t="s">
+      <c r="F13" s="44">
+        <f>$F11*E13</f>
+        <v>1776.5000000000007</v>
+      </c>
+      <c r="G13" s="37"/>
+    </row>
+    <row r="14" spans="1:8" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B14" s="63" t="s">
+        <v>67</v>
+      </c>
+      <c r="C14" s="161" t="s">
+        <v>93</v>
+      </c>
+      <c r="D14" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="E14" s="151">
+        <v>1</v>
+      </c>
+      <c r="F14" s="44">
+        <f>$F11*E14</f>
+        <v>1615.0000000000005</v>
+      </c>
+      <c r="G14" s="37"/>
+    </row>
+    <row r="15" spans="1:8" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="B15" s="63" t="s">
+        <v>95</v>
+      </c>
+      <c r="C15" s="161" t="s">
+        <v>99</v>
+      </c>
+      <c r="D15" s="67" t="s">
         <v>72</v>
       </c>
-      <c r="F7" s="37"/>
-    </row>
-    <row r="8" spans="1:7" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B8" s="73" t="s">
-        <v>62</v>
-      </c>
-      <c r="C8" s="75" t="s">
-        <v>75</v>
-      </c>
-      <c r="D8" s="16">
-        <f>D6*1.1</f>
-        <v>1090.9470000000001</v>
-      </c>
-      <c r="E8" s="44" t="s">
-        <v>69</v>
-      </c>
-      <c r="F8" s="37"/>
-    </row>
-    <row r="9" spans="1:7" s="13" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="74" t="s">
-        <v>63</v>
-      </c>
-      <c r="C9" s="80" t="s">
-        <v>71</v>
-      </c>
-      <c r="D9" s="76">
-        <f>D6*0.25</f>
-        <v>247.9425</v>
-      </c>
-      <c r="E9" s="46" t="s">
-        <v>72</v>
-      </c>
-      <c r="F9" s="37"/>
-    </row>
-    <row r="10" spans="1:7" s="13" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="B10" s="77" t="s">
-        <v>64</v>
-      </c>
-      <c r="C10" s="98" t="s">
-        <v>74</v>
-      </c>
-      <c r="D10" s="79">
-        <f>D5-D6</f>
-        <v>1615.0000000000005</v>
-      </c>
-      <c r="E10" s="47" t="s">
-        <v>69</v>
-      </c>
-      <c r="F10" s="37"/>
-    </row>
-    <row r="11" spans="1:7" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B11" s="73" t="s">
-        <v>66</v>
-      </c>
-      <c r="C11" s="75" t="s">
-        <v>76</v>
-      </c>
-      <c r="D11" s="16">
-        <f>D10*1.3</f>
-        <v>2099.5000000000005</v>
-      </c>
-      <c r="E11" s="44" t="s">
-        <v>72</v>
-      </c>
-      <c r="F11" s="37"/>
-    </row>
-    <row r="12" spans="1:7" s="13" customFormat="1" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="B12" s="73" t="s">
-        <v>65</v>
-      </c>
-      <c r="C12" s="75" t="s">
-        <v>75</v>
-      </c>
-      <c r="D12" s="16">
-        <f>D10</f>
-        <v>1615.0000000000005</v>
-      </c>
-      <c r="E12" s="44" t="s">
-        <v>69</v>
-      </c>
-      <c r="F12" s="37"/>
-    </row>
-    <row r="13" spans="1:7" s="13" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="74" t="s">
-        <v>67</v>
-      </c>
-      <c r="C13" s="80" t="s">
-        <v>60</v>
-      </c>
-      <c r="D13" s="76">
-        <f>D10*0.25</f>
-        <v>403.75000000000011</v>
-      </c>
-      <c r="E13" s="46" t="s">
-        <v>72</v>
-      </c>
-      <c r="F13" s="37"/>
-    </row>
-    <row r="14" spans="1:7" s="13" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="85">
-        <v>2</v>
-      </c>
-      <c r="C14" s="86" t="s">
-        <v>57</v>
-      </c>
-      <c r="D14" s="87">
-        <f>D12+D8</f>
-        <v>2705.9470000000006</v>
-      </c>
-      <c r="E14" s="88" t="s">
-        <v>69</v>
-      </c>
-      <c r="F14" s="37"/>
-    </row>
-    <row r="15" spans="1:7" s="13" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="81">
-        <v>3</v>
-      </c>
-      <c r="C15" s="82" t="s">
+      <c r="E15" s="151">
+        <f>E11*0.15</f>
+        <v>0.15</v>
+      </c>
+      <c r="F15" s="44">
+        <f>$F11*E15</f>
+        <v>242.25000000000006</v>
+      </c>
+      <c r="G15" s="37"/>
+    </row>
+    <row r="16" spans="1:8" s="13" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="64" t="s">
+        <v>83</v>
+      </c>
+      <c r="C16" s="154" t="s">
         <v>11</v>
       </c>
-      <c r="D15" s="83">
+      <c r="D16" s="65" t="s">
+        <v>70</v>
+      </c>
+      <c r="E16" s="153">
+        <v>1</v>
+      </c>
+      <c r="F16" s="46">
         <v>717.45</v>
       </c>
-      <c r="E15" s="84" t="s">
-        <v>70</v>
-      </c>
-      <c r="F15" s="37"/>
+      <c r="G16" s="37"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4123,906 +4134,906 @@
   <dimension ref="B2:H78"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="152"/>
-    <col min="2" max="2" width="7" style="152" customWidth="1"/>
-    <col min="3" max="3" width="10" style="152" customWidth="1"/>
-    <col min="4" max="4" width="56.85546875" style="152" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.28515625" style="152" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.5703125" style="152" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="9.140625" style="152"/>
+    <col min="1" max="1" width="9.140625" style="115"/>
+    <col min="2" max="2" width="7" style="115" customWidth="1"/>
+    <col min="3" max="3" width="10" style="115" customWidth="1"/>
+    <col min="4" max="4" width="56.85546875" style="115" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.28515625" style="115" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" style="115" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="115"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="3" spans="2:8" s="105" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="153"/>
-      <c r="C3" s="154"/>
-      <c r="D3" s="155" t="s">
+    <row r="3" spans="2:8" s="80" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="116"/>
+      <c r="C3" s="117"/>
+      <c r="D3" s="118" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="156"/>
-      <c r="F3" s="157"/>
-      <c r="G3" s="158"/>
-    </row>
-    <row r="4" spans="2:8" s="105" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="159" t="s">
+      <c r="E3" s="119"/>
+      <c r="F3" s="120"/>
+      <c r="G3" s="121"/>
+    </row>
+    <row r="4" spans="2:8" s="80" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="122" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="160" t="s">
+      <c r="C4" s="123" t="s">
         <v>58</v>
       </c>
-      <c r="D4" s="161" t="s">
+      <c r="D4" s="124" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="135" t="s">
+      <c r="E4" s="108" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="157"/>
-      <c r="G4" s="158"/>
-    </row>
-    <row r="5" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="162">
-        <v>1</v>
-      </c>
-      <c r="C5" s="163" t="s">
+      <c r="F4" s="120"/>
+      <c r="G4" s="121"/>
+    </row>
+    <row r="5" spans="2:8" s="80" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="125">
+        <v>1</v>
+      </c>
+      <c r="C5" s="126" t="s">
         <v>54</v>
       </c>
-      <c r="D5" s="164" t="s">
+      <c r="D5" s="127" t="s">
         <v>78</v>
       </c>
-      <c r="E5" s="165">
+      <c r="E5" s="128">
         <v>336.4</v>
       </c>
-      <c r="F5" s="157"/>
-      <c r="G5" s="158"/>
-    </row>
-    <row r="6" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="166"/>
-      <c r="C6" s="167"/>
-      <c r="D6" s="140" t="s">
-        <v>1</v>
-      </c>
-      <c r="E6" s="126">
+      <c r="F5" s="120"/>
+      <c r="G5" s="121"/>
+    </row>
+    <row r="6" spans="2:8" s="80" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="129"/>
+      <c r="C6" s="130"/>
+      <c r="D6" s="113" t="s">
+        <v>1</v>
+      </c>
+      <c r="E6" s="99">
         <v>30.2</v>
       </c>
-      <c r="F6" s="157"/>
-      <c r="G6" s="158"/>
-      <c r="H6" s="158">
+      <c r="F6" s="120"/>
+      <c r="G6" s="121"/>
+      <c r="H6" s="121">
         <f>E6</f>
         <v>30.2</v>
       </c>
     </row>
-    <row r="7" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="166"/>
-      <c r="C7" s="167"/>
-      <c r="D7" s="140" t="s">
+    <row r="7" spans="2:8" s="80" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="129"/>
+      <c r="C7" s="130"/>
+      <c r="D7" s="113" t="s">
         <v>57</v>
       </c>
-      <c r="E7" s="126">
+      <c r="E7" s="99">
         <f>E6</f>
         <v>30.2</v>
       </c>
-      <c r="F7" s="157"/>
-      <c r="G7" s="158"/>
-    </row>
-    <row r="8" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="166"/>
-      <c r="C8" s="167"/>
-      <c r="D8" s="168" t="s">
+      <c r="F7" s="120"/>
+      <c r="G7" s="121"/>
+    </row>
+    <row r="8" spans="2:8" s="80" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="129"/>
+      <c r="C8" s="130"/>
+      <c r="D8" s="131" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="169" t="str">
+      <c r="E8" s="132" t="str">
         <f>TEXT(G8, "0.00") &amp; " п.м"</f>
         <v>60.41 п.м</v>
       </c>
-      <c r="F8" s="157"/>
-      <c r="G8" s="158">
+      <c r="F8" s="120"/>
+      <c r="G8" s="121">
         <v>60.41</v>
       </c>
     </row>
-    <row r="9" spans="2:8" s="105" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="170"/>
-      <c r="C9" s="171"/>
-      <c r="D9" s="172" t="s">
+    <row r="9" spans="2:8" s="80" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="133"/>
+      <c r="C9" s="134"/>
+      <c r="D9" s="135" t="s">
         <v>81</v>
       </c>
-      <c r="E9" s="130">
+      <c r="E9" s="103">
         <f>E5</f>
         <v>336.4</v>
       </c>
-      <c r="F9" s="157"/>
-      <c r="G9" s="158"/>
-    </row>
-    <row r="10" spans="2:8" s="105" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="153"/>
-      <c r="C10" s="154"/>
-      <c r="D10" s="155" t="s">
+      <c r="F9" s="120"/>
+      <c r="G9" s="121"/>
+    </row>
+    <row r="10" spans="2:8" s="80" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="116"/>
+      <c r="C10" s="117"/>
+      <c r="D10" s="118" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="156"/>
-      <c r="F10" s="157"/>
-      <c r="G10" s="158"/>
-    </row>
-    <row r="11" spans="2:8" s="105" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="159" t="s">
+      <c r="E10" s="119"/>
+      <c r="F10" s="120"/>
+      <c r="G10" s="121"/>
+    </row>
+    <row r="11" spans="2:8" s="80" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="122" t="s">
         <v>6</v>
       </c>
-      <c r="C11" s="160" t="s">
+      <c r="C11" s="123" t="s">
         <v>58</v>
       </c>
-      <c r="D11" s="161" t="s">
+      <c r="D11" s="124" t="s">
         <v>7</v>
       </c>
-      <c r="E11" s="135" t="s">
+      <c r="E11" s="108" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="157"/>
-      <c r="G11" s="158"/>
-    </row>
-    <row r="12" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="173">
+      <c r="F11" s="120"/>
+      <c r="G11" s="121"/>
+    </row>
+    <row r="12" spans="2:8" s="80" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B12" s="136">
         <v>2</v>
       </c>
-      <c r="C12" s="174" t="s">
+      <c r="C12" s="137" t="s">
         <v>77</v>
       </c>
-      <c r="D12" s="175" t="s">
+      <c r="D12" s="138" t="s">
         <v>78</v>
       </c>
-      <c r="E12" s="123">
+      <c r="E12" s="96">
         <v>543.35</v>
       </c>
-      <c r="F12" s="157"/>
-      <c r="G12" s="158"/>
-    </row>
-    <row r="13" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="166"/>
-      <c r="C13" s="167"/>
-      <c r="D13" s="140" t="s">
-        <v>1</v>
-      </c>
-      <c r="E13" s="126">
+      <c r="F12" s="120"/>
+      <c r="G12" s="121"/>
+    </row>
+    <row r="13" spans="2:8" s="80" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="129"/>
+      <c r="C13" s="130"/>
+      <c r="D13" s="113" t="s">
+        <v>1</v>
+      </c>
+      <c r="E13" s="99">
         <v>28.32</v>
       </c>
-      <c r="F13" s="157"/>
-      <c r="G13" s="158"/>
-      <c r="H13" s="158">
+      <c r="F13" s="120"/>
+      <c r="G13" s="121"/>
+      <c r="H13" s="121">
         <f>E13</f>
         <v>28.32</v>
       </c>
     </row>
-    <row r="14" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="166"/>
-      <c r="C14" s="167"/>
-      <c r="D14" s="140" t="s">
+    <row r="14" spans="2:8" s="80" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="129"/>
+      <c r="C14" s="130"/>
+      <c r="D14" s="113" t="s">
         <v>57</v>
       </c>
-      <c r="E14" s="126">
+      <c r="E14" s="99">
         <f>E13</f>
         <v>28.32</v>
       </c>
-      <c r="F14" s="157"/>
-      <c r="G14" s="158"/>
-    </row>
-    <row r="15" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="166"/>
-      <c r="C15" s="167"/>
-      <c r="D15" s="168" t="s">
+      <c r="F14" s="120"/>
+      <c r="G14" s="121"/>
+    </row>
+    <row r="15" spans="2:8" s="80" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="129"/>
+      <c r="C15" s="130"/>
+      <c r="D15" s="131" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="169" t="str">
+      <c r="E15" s="132" t="str">
         <f>TEXT(G15, "0.00") &amp; " п.м"</f>
         <v>51.28 п.м</v>
       </c>
-      <c r="F15" s="157"/>
-      <c r="G15" s="158">
+      <c r="F15" s="120"/>
+      <c r="G15" s="121">
         <v>51.28</v>
       </c>
     </row>
-    <row r="16" spans="2:8" s="105" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="170"/>
-      <c r="C16" s="171"/>
-      <c r="D16" s="172" t="s">
+    <row r="16" spans="2:8" s="80" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="133"/>
+      <c r="C16" s="134"/>
+      <c r="D16" s="135" t="s">
         <v>81</v>
       </c>
-      <c r="E16" s="130">
+      <c r="E16" s="103">
         <f>E12</f>
         <v>543.35</v>
       </c>
-      <c r="F16" s="157"/>
-      <c r="G16" s="158"/>
-    </row>
-    <row r="17" spans="2:7" s="105" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="106"/>
-      <c r="C17" s="176"/>
-      <c r="D17" s="177"/>
-      <c r="E17" s="178"/>
-      <c r="F17" s="157"/>
-      <c r="G17" s="158"/>
-    </row>
-    <row r="18" spans="2:7" s="105" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="106"/>
-      <c r="C18" s="176"/>
-      <c r="D18" s="177"/>
-      <c r="E18" s="178"/>
-      <c r="F18" s="157"/>
-      <c r="G18" s="158"/>
-    </row>
-    <row r="19" spans="2:7" s="105" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="153"/>
-      <c r="C19" s="154"/>
-      <c r="D19" s="155" t="s">
+      <c r="F16" s="120"/>
+      <c r="G16" s="121"/>
+    </row>
+    <row r="17" spans="2:7" s="80" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B17" s="81"/>
+      <c r="C17" s="139"/>
+      <c r="D17" s="140"/>
+      <c r="E17" s="141"/>
+      <c r="F17" s="120"/>
+      <c r="G17" s="121"/>
+    </row>
+    <row r="18" spans="2:7" s="80" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="81"/>
+      <c r="C18" s="139"/>
+      <c r="D18" s="140"/>
+      <c r="E18" s="141"/>
+      <c r="F18" s="120"/>
+      <c r="G18" s="121"/>
+    </row>
+    <row r="19" spans="2:7" s="80" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="116"/>
+      <c r="C19" s="117"/>
+      <c r="D19" s="118" t="s">
         <v>9</v>
       </c>
-      <c r="E19" s="156"/>
-      <c r="F19" s="157"/>
-      <c r="G19" s="158"/>
-    </row>
-    <row r="20" spans="2:7" s="105" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="159" t="s">
+      <c r="E19" s="119"/>
+      <c r="F19" s="120"/>
+      <c r="G19" s="121"/>
+    </row>
+    <row r="20" spans="2:7" s="80" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="122" t="s">
         <v>6</v>
       </c>
-      <c r="C20" s="160" t="s">
+      <c r="C20" s="123" t="s">
         <v>58</v>
       </c>
-      <c r="D20" s="161" t="s">
+      <c r="D20" s="124" t="s">
         <v>7</v>
       </c>
-      <c r="E20" s="135" t="s">
+      <c r="E20" s="108" t="s">
         <v>28</v>
       </c>
-      <c r="F20" s="157"/>
-      <c r="G20" s="158"/>
-    </row>
-    <row r="21" spans="2:7" s="105" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="B21" s="173">
+      <c r="F20" s="120"/>
+      <c r="G20" s="121"/>
+    </row>
+    <row r="21" spans="2:7" s="80" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="B21" s="136">
         <v>3</v>
       </c>
-      <c r="C21" s="179" t="s">
+      <c r="C21" s="142" t="s">
         <v>79</v>
       </c>
-      <c r="D21" s="175" t="s">
+      <c r="D21" s="138" t="s">
         <v>78</v>
       </c>
-      <c r="E21" s="123">
+      <c r="E21" s="96">
         <v>196.34</v>
       </c>
-      <c r="F21" s="157"/>
-      <c r="G21" s="158"/>
-    </row>
-    <row r="22" spans="2:7" s="105" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="170"/>
-      <c r="C22" s="180"/>
-      <c r="D22" s="172" t="s">
+      <c r="F21" s="120"/>
+      <c r="G21" s="121"/>
+    </row>
+    <row r="22" spans="2:7" s="80" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="133"/>
+      <c r="C22" s="143"/>
+      <c r="D22" s="135" t="s">
         <v>81</v>
       </c>
-      <c r="E22" s="130">
+      <c r="E22" s="103">
         <f>E21</f>
         <v>196.34</v>
       </c>
-      <c r="F22" s="157"/>
-      <c r="G22" s="158"/>
-    </row>
-    <row r="23" spans="2:7" s="105" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="106"/>
-      <c r="C23" s="176"/>
-      <c r="D23" s="177"/>
-      <c r="E23" s="178"/>
-      <c r="F23" s="157"/>
-      <c r="G23" s="158"/>
-    </row>
-    <row r="24" spans="2:7" s="105" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="106"/>
-      <c r="C24" s="176"/>
-      <c r="D24" s="177"/>
-      <c r="E24" s="178"/>
-      <c r="F24" s="157"/>
-      <c r="G24" s="158"/>
-    </row>
-    <row r="25" spans="2:7" s="105" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="153"/>
-      <c r="C25" s="154"/>
-      <c r="D25" s="155" t="s">
+      <c r="F22" s="120"/>
+      <c r="G22" s="121"/>
+    </row>
+    <row r="23" spans="2:7" s="80" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B23" s="81"/>
+      <c r="C23" s="139"/>
+      <c r="D23" s="140"/>
+      <c r="E23" s="141"/>
+      <c r="F23" s="120"/>
+      <c r="G23" s="121"/>
+    </row>
+    <row r="24" spans="2:7" s="80" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="81"/>
+      <c r="C24" s="139"/>
+      <c r="D24" s="140"/>
+      <c r="E24" s="141"/>
+      <c r="F24" s="120"/>
+      <c r="G24" s="121"/>
+    </row>
+    <row r="25" spans="2:7" s="80" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="116"/>
+      <c r="C25" s="117"/>
+      <c r="D25" s="118" t="s">
         <v>9</v>
       </c>
-      <c r="E25" s="156"/>
-      <c r="F25" s="157"/>
-      <c r="G25" s="158"/>
-    </row>
-    <row r="26" spans="2:7" s="105" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="159" t="s">
+      <c r="E25" s="119"/>
+      <c r="F25" s="120"/>
+      <c r="G25" s="121"/>
+    </row>
+    <row r="26" spans="2:7" s="80" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="122" t="s">
         <v>6</v>
       </c>
-      <c r="C26" s="160" t="s">
+      <c r="C26" s="123" t="s">
         <v>58</v>
       </c>
-      <c r="D26" s="161" t="s">
+      <c r="D26" s="124" t="s">
         <v>7</v>
       </c>
-      <c r="E26" s="135" t="s">
+      <c r="E26" s="108" t="s">
         <v>28</v>
       </c>
-      <c r="F26" s="157"/>
-      <c r="G26" s="158"/>
-    </row>
-    <row r="27" spans="2:7" s="105" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B27" s="173">
+      <c r="F26" s="120"/>
+      <c r="G26" s="121"/>
+    </row>
+    <row r="27" spans="2:7" s="80" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="136">
         <v>4</v>
       </c>
-      <c r="C27" s="179" t="s">
+      <c r="C27" s="142" t="s">
         <v>56</v>
       </c>
-      <c r="D27" s="175" t="s">
+      <c r="D27" s="138" t="s">
         <v>78</v>
       </c>
-      <c r="E27" s="123">
+      <c r="E27" s="96">
         <v>192.38</v>
       </c>
-      <c r="F27" s="157"/>
-      <c r="G27" s="158"/>
-    </row>
-    <row r="28" spans="2:7" s="105" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="170"/>
-      <c r="C28" s="180"/>
-      <c r="D28" s="172" t="s">
+      <c r="F27" s="120"/>
+      <c r="G27" s="121"/>
+    </row>
+    <row r="28" spans="2:7" s="80" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="133"/>
+      <c r="C28" s="143"/>
+      <c r="D28" s="135" t="s">
         <v>81</v>
       </c>
-      <c r="E28" s="130">
+      <c r="E28" s="103">
         <f>E27</f>
         <v>192.38</v>
       </c>
-      <c r="F28" s="157"/>
-      <c r="G28" s="158"/>
-    </row>
-    <row r="29" spans="2:7" s="105" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="106"/>
-      <c r="C29" s="176"/>
-      <c r="D29" s="177"/>
-      <c r="E29" s="178"/>
-      <c r="F29" s="157"/>
-      <c r="G29" s="158"/>
-    </row>
-    <row r="30" spans="2:7" s="105" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="106"/>
-      <c r="C30" s="176"/>
-      <c r="D30" s="177"/>
-      <c r="E30" s="178"/>
-      <c r="F30" s="157"/>
-      <c r="G30" s="158"/>
-    </row>
-    <row r="31" spans="2:7" s="105" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="106"/>
-      <c r="C31" s="176"/>
-      <c r="D31" s="177"/>
-      <c r="E31" s="178"/>
-      <c r="F31" s="157"/>
-      <c r="G31" s="158"/>
-    </row>
-    <row r="32" spans="2:7" s="105" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="181"/>
-      <c r="C32" s="103" t="s">
+      <c r="F28" s="120"/>
+      <c r="G28" s="121"/>
+    </row>
+    <row r="29" spans="2:7" s="80" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="81"/>
+      <c r="C29" s="139"/>
+      <c r="D29" s="140"/>
+      <c r="E29" s="141"/>
+      <c r="F29" s="120"/>
+      <c r="G29" s="121"/>
+    </row>
+    <row r="30" spans="2:7" s="80" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="81"/>
+      <c r="C30" s="139"/>
+      <c r="D30" s="140"/>
+      <c r="E30" s="141"/>
+      <c r="F30" s="120"/>
+      <c r="G30" s="121"/>
+    </row>
+    <row r="31" spans="2:7" s="80" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="81"/>
+      <c r="C31" s="139"/>
+      <c r="D31" s="140"/>
+      <c r="E31" s="141"/>
+      <c r="F31" s="120"/>
+      <c r="G31" s="121"/>
+    </row>
+    <row r="32" spans="2:7" s="80" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="144"/>
+      <c r="C32" s="79" t="s">
         <v>6</v>
       </c>
-      <c r="D32" s="140" t="s">
+      <c r="D32" s="113" t="s">
         <v>7</v>
       </c>
-      <c r="E32" s="125" t="s">
+      <c r="E32" s="98" t="s">
         <v>28</v>
       </c>
-      <c r="F32" s="157"/>
-    </row>
-    <row r="33" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="181"/>
-      <c r="C33" s="103">
-        <v>1</v>
-      </c>
-      <c r="D33" s="140" t="s">
+      <c r="F32" s="120"/>
+    </row>
+    <row r="33" spans="2:8" s="80" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="144"/>
+      <c r="C33" s="79">
+        <v>1</v>
+      </c>
+      <c r="D33" s="113" t="s">
         <v>12</v>
       </c>
-      <c r="E33" s="125">
+      <c r="E33" s="98">
         <v>340.88</v>
       </c>
-      <c r="F33" s="157"/>
-    </row>
-    <row r="34" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B34" s="181"/>
-      <c r="C34" s="103">
+      <c r="F33" s="120"/>
+    </row>
+    <row r="34" spans="2:8" s="80" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="144"/>
+      <c r="C34" s="79">
         <v>2</v>
       </c>
-      <c r="D34" s="140" t="s">
+      <c r="D34" s="113" t="s">
         <v>13</v>
       </c>
-      <c r="E34" s="125">
+      <c r="E34" s="98">
         <v>0</v>
       </c>
-      <c r="F34" s="157"/>
-    </row>
-    <row r="35" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="181"/>
-      <c r="C35" s="103">
+      <c r="F34" s="120"/>
+    </row>
+    <row r="35" spans="2:8" s="80" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="144"/>
+      <c r="C35" s="79">
         <v>3</v>
       </c>
-      <c r="D35" s="140" t="s">
+      <c r="D35" s="113" t="s">
         <v>36</v>
       </c>
-      <c r="E35" s="125">
+      <c r="E35" s="98">
         <v>340.88</v>
       </c>
-      <c r="F35" s="157"/>
-    </row>
-    <row r="36" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B36" s="181"/>
-      <c r="C36" s="103">
+      <c r="F35" s="120"/>
+    </row>
+    <row r="36" spans="2:8" s="80" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B36" s="144"/>
+      <c r="C36" s="79">
         <v>4</v>
       </c>
-      <c r="D36" s="140" t="s">
+      <c r="D36" s="113" t="s">
         <v>35</v>
       </c>
-      <c r="E36" s="125">
+      <c r="E36" s="98">
         <v>0</v>
       </c>
-      <c r="F36" s="157"/>
-    </row>
-    <row r="37" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B37" s="181"/>
-      <c r="C37" s="103">
+      <c r="F36" s="120"/>
+    </row>
+    <row r="37" spans="2:8" s="80" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B37" s="144"/>
+      <c r="C37" s="79">
         <v>5</v>
       </c>
-      <c r="D37" s="140" t="s">
+      <c r="D37" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="E37" s="125" t="s">
+      <c r="E37" s="98" t="s">
         <v>26</v>
       </c>
-      <c r="F37" s="157"/>
-      <c r="H37" s="158"/>
-    </row>
-    <row r="38" spans="2:8" s="105" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B38" s="181"/>
-      <c r="C38" s="103">
+      <c r="F37" s="120"/>
+      <c r="H37" s="121"/>
+    </row>
+    <row r="38" spans="2:8" s="80" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B38" s="144"/>
+      <c r="C38" s="79">
         <v>6</v>
       </c>
-      <c r="D38" s="124"/>
-      <c r="E38" s="125">
+      <c r="D38" s="97"/>
+      <c r="E38" s="98">
         <f>E33</f>
         <v>340.88</v>
       </c>
-      <c r="F38" s="157"/>
+      <c r="F38" s="120"/>
     </row>
     <row r="40" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="41" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B41" s="153"/>
-      <c r="C41" s="154"/>
-      <c r="D41" s="155"/>
-      <c r="E41" s="156"/>
+      <c r="B41" s="116"/>
+      <c r="C41" s="117"/>
+      <c r="D41" s="118"/>
+      <c r="E41" s="119"/>
     </row>
     <row r="42" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B42" s="159" t="s">
+      <c r="B42" s="122" t="s">
         <v>6</v>
       </c>
-      <c r="C42" s="160" t="s">
+      <c r="C42" s="123" t="s">
         <v>58</v>
       </c>
-      <c r="D42" s="161" t="s">
+      <c r="D42" s="124" t="s">
         <v>7</v>
       </c>
-      <c r="E42" s="135" t="s">
+      <c r="E42" s="108" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="43" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B43" s="162"/>
-      <c r="C43" s="163"/>
-      <c r="D43" s="164" t="s">
+      <c r="B43" s="125"/>
+      <c r="C43" s="126"/>
+      <c r="D43" s="127" t="s">
         <v>78</v>
       </c>
-      <c r="E43" s="165">
+      <c r="E43" s="128">
         <f>E5+E12+E21+E27</f>
         <v>1268.4699999999998</v>
       </c>
     </row>
     <row r="44" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B44" s="166"/>
-      <c r="C44" s="167"/>
-      <c r="D44" s="140" t="s">
-        <v>1</v>
-      </c>
-      <c r="E44" s="126">
+      <c r="B44" s="129"/>
+      <c r="C44" s="130"/>
+      <c r="D44" s="113" t="s">
+        <v>1</v>
+      </c>
+      <c r="E44" s="99">
         <f>E13+E6</f>
         <v>58.519999999999996</v>
       </c>
     </row>
     <row r="45" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B45" s="166"/>
-      <c r="C45" s="167"/>
-      <c r="D45" s="140" t="s">
+      <c r="B45" s="129"/>
+      <c r="C45" s="130"/>
+      <c r="D45" s="113" t="s">
         <v>57</v>
       </c>
-      <c r="E45" s="126">
+      <c r="E45" s="99">
         <f>E44</f>
         <v>58.519999999999996</v>
       </c>
     </row>
     <row r="46" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B46" s="166"/>
-      <c r="C46" s="167"/>
-      <c r="D46" s="168" t="s">
+      <c r="B46" s="129"/>
+      <c r="C46" s="130"/>
+      <c r="D46" s="131" t="s">
         <v>11</v>
       </c>
-      <c r="E46" s="169" t="str">
+      <c r="E46" s="132" t="str">
         <f>TEXT(G46, "0.00") &amp; " п.м"</f>
         <v>111.69 п.м</v>
       </c>
-      <c r="G46" s="182">
+      <c r="G46" s="145">
         <f>G15+G8</f>
         <v>111.69</v>
       </c>
     </row>
     <row r="47" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="170"/>
-      <c r="C47" s="171"/>
-      <c r="D47" s="172" t="s">
+      <c r="B47" s="133"/>
+      <c r="C47" s="134"/>
+      <c r="D47" s="135" t="s">
         <v>12</v>
       </c>
-      <c r="E47" s="130">
+      <c r="E47" s="103">
         <f>E43</f>
         <v>1268.4699999999998</v>
       </c>
     </row>
     <row r="49" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="50" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B50" s="153"/>
-      <c r="C50" s="154"/>
-      <c r="D50" s="155" t="s">
+      <c r="B50" s="116"/>
+      <c r="C50" s="117"/>
+      <c r="D50" s="118" t="s">
         <v>9</v>
       </c>
-      <c r="E50" s="156"/>
+      <c r="E50" s="119"/>
     </row>
     <row r="51" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B51" s="159" t="s">
+      <c r="B51" s="122" t="s">
         <v>6</v>
       </c>
-      <c r="C51" s="160" t="s">
+      <c r="C51" s="123" t="s">
         <v>58</v>
       </c>
-      <c r="D51" s="161" t="s">
+      <c r="D51" s="124" t="s">
         <v>7</v>
       </c>
-      <c r="E51" s="135" t="s">
+      <c r="E51" s="108" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="52" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B52" s="162">
-        <v>1</v>
-      </c>
-      <c r="C52" s="163" t="s">
+      <c r="B52" s="125">
+        <v>1</v>
+      </c>
+      <c r="C52" s="126" t="s">
         <v>54</v>
       </c>
-      <c r="D52" s="164" t="s">
+      <c r="D52" s="127" t="s">
         <v>78</v>
       </c>
-      <c r="E52" s="165">
+      <c r="E52" s="128">
         <v>336.4</v>
       </c>
     </row>
     <row r="53" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B53" s="166"/>
-      <c r="C53" s="167"/>
-      <c r="D53" s="140" t="s">
-        <v>1</v>
-      </c>
-      <c r="E53" s="126">
+      <c r="B53" s="129"/>
+      <c r="C53" s="130"/>
+      <c r="D53" s="113" t="s">
+        <v>1</v>
+      </c>
+      <c r="E53" s="99">
         <v>30.2</v>
       </c>
     </row>
     <row r="54" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B54" s="166"/>
-      <c r="C54" s="167"/>
-      <c r="D54" s="140" t="s">
+      <c r="B54" s="129"/>
+      <c r="C54" s="130"/>
+      <c r="D54" s="113" t="s">
         <v>57</v>
       </c>
-      <c r="E54" s="126">
+      <c r="E54" s="99">
         <f>E53</f>
         <v>30.2</v>
       </c>
     </row>
     <row r="55" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B55" s="166"/>
-      <c r="C55" s="167"/>
-      <c r="D55" s="168" t="s">
+      <c r="B55" s="129"/>
+      <c r="C55" s="130"/>
+      <c r="D55" s="131" t="s">
         <v>11</v>
       </c>
-      <c r="E55" s="169" t="str">
+      <c r="E55" s="132" t="str">
         <f>TEXT(G55, "0.00") &amp; " п.м"</f>
         <v>60.41 п.м</v>
       </c>
-      <c r="G55" s="158">
+      <c r="G55" s="121">
         <v>60.41</v>
       </c>
     </row>
     <row r="56" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="170"/>
-      <c r="C56" s="171"/>
-      <c r="D56" s="172" t="s">
+      <c r="B56" s="133"/>
+      <c r="C56" s="134"/>
+      <c r="D56" s="135" t="s">
         <v>81</v>
       </c>
-      <c r="E56" s="130">
+      <c r="E56" s="103">
         <f>E52</f>
         <v>336.4</v>
       </c>
-      <c r="G56" s="158"/>
+      <c r="G56" s="121"/>
     </row>
     <row r="57" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B57" s="173">
+      <c r="B57" s="136">
         <v>2</v>
       </c>
-      <c r="C57" s="174" t="s">
+      <c r="C57" s="137" t="s">
         <v>77</v>
       </c>
-      <c r="D57" s="175" t="s">
+      <c r="D57" s="138" t="s">
         <v>78</v>
       </c>
-      <c r="E57" s="123">
+      <c r="E57" s="96">
         <v>543.35</v>
       </c>
-      <c r="G57" s="158"/>
+      <c r="G57" s="121"/>
     </row>
     <row r="58" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B58" s="166"/>
-      <c r="C58" s="167"/>
-      <c r="D58" s="140" t="s">
-        <v>1</v>
-      </c>
-      <c r="E58" s="126">
+      <c r="B58" s="129"/>
+      <c r="C58" s="130"/>
+      <c r="D58" s="113" t="s">
+        <v>1</v>
+      </c>
+      <c r="E58" s="99">
         <v>28.32</v>
       </c>
-      <c r="G58" s="158"/>
+      <c r="G58" s="121"/>
     </row>
     <row r="59" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B59" s="166"/>
-      <c r="C59" s="167"/>
-      <c r="D59" s="140" t="s">
+      <c r="B59" s="129"/>
+      <c r="C59" s="130"/>
+      <c r="D59" s="113" t="s">
         <v>57</v>
       </c>
-      <c r="E59" s="126">
+      <c r="E59" s="99">
         <f>E58</f>
         <v>28.32</v>
       </c>
-      <c r="G59" s="158"/>
+      <c r="G59" s="121"/>
     </row>
     <row r="60" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B60" s="166"/>
-      <c r="C60" s="167"/>
-      <c r="D60" s="168" t="s">
+      <c r="B60" s="129"/>
+      <c r="C60" s="130"/>
+      <c r="D60" s="131" t="s">
         <v>11</v>
       </c>
-      <c r="E60" s="169" t="str">
+      <c r="E60" s="132" t="str">
         <f>TEXT(G60, "0.00") &amp; " п.м"</f>
         <v>51.28 п.м</v>
       </c>
-      <c r="G60" s="158">
+      <c r="G60" s="121">
         <v>51.28</v>
       </c>
     </row>
     <row r="61" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B61" s="170"/>
-      <c r="C61" s="171"/>
-      <c r="D61" s="172" t="s">
+      <c r="B61" s="133"/>
+      <c r="C61" s="134"/>
+      <c r="D61" s="135" t="s">
         <v>81</v>
       </c>
-      <c r="E61" s="130">
+      <c r="E61" s="103">
         <f>E57</f>
         <v>543.35</v>
       </c>
-      <c r="G61" s="158"/>
+      <c r="G61" s="121"/>
     </row>
     <row r="62" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B62" s="173">
+      <c r="B62" s="136">
         <v>3</v>
       </c>
-      <c r="C62" s="179" t="s">
+      <c r="C62" s="142" t="s">
         <v>47</v>
       </c>
-      <c r="D62" s="175" t="s">
+      <c r="D62" s="138" t="s">
         <v>78</v>
       </c>
-      <c r="E62" s="123">
+      <c r="E62" s="96">
         <v>143.85999999999999</v>
       </c>
-      <c r="F62" s="182">
+      <c r="F62" s="145">
         <f>E62</f>
         <v>143.85999999999999</v>
       </c>
     </row>
     <row r="63" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B63" s="170"/>
-      <c r="C63" s="180"/>
-      <c r="D63" s="172" t="s">
+      <c r="B63" s="133"/>
+      <c r="C63" s="143"/>
+      <c r="D63" s="135" t="s">
         <v>81</v>
       </c>
-      <c r="E63" s="130">
+      <c r="E63" s="103">
         <f>E62</f>
         <v>143.85999999999999</v>
       </c>
     </row>
     <row r="64" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B64" s="173">
+      <c r="B64" s="136">
         <v>4</v>
       </c>
-      <c r="C64" s="179" t="s">
-        <v>94</v>
-      </c>
-      <c r="D64" s="175" t="s">
+      <c r="C64" s="142" t="s">
+        <v>88</v>
+      </c>
+      <c r="D64" s="138" t="s">
         <v>78</v>
       </c>
-      <c r="E64" s="123">
+      <c r="E64" s="96">
         <v>5.24</v>
       </c>
-      <c r="F64" s="182">
+      <c r="F64" s="145">
         <f>E64</f>
         <v>5.24</v>
       </c>
     </row>
     <row r="65" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B65" s="170"/>
-      <c r="C65" s="180"/>
-      <c r="D65" s="172" t="s">
+      <c r="B65" s="133"/>
+      <c r="C65" s="143"/>
+      <c r="D65" s="135" t="s">
         <v>81</v>
       </c>
-      <c r="E65" s="130">
+      <c r="E65" s="103">
         <f>E64</f>
         <v>5.24</v>
       </c>
     </row>
     <row r="66" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B66" s="173">
+      <c r="B66" s="136">
         <v>5</v>
       </c>
-      <c r="C66" s="179" t="s">
-        <v>95</v>
-      </c>
-      <c r="D66" s="175" t="s">
+      <c r="C66" s="142" t="s">
+        <v>89</v>
+      </c>
+      <c r="D66" s="138" t="s">
         <v>78</v>
       </c>
-      <c r="E66" s="123">
+      <c r="E66" s="96">
         <v>12.32</v>
       </c>
-      <c r="F66" s="182">
+      <c r="F66" s="145">
         <f>E66</f>
         <v>12.32</v>
       </c>
     </row>
     <row r="67" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B67" s="170"/>
-      <c r="C67" s="180"/>
-      <c r="D67" s="172" t="s">
+      <c r="B67" s="133"/>
+      <c r="C67" s="143"/>
+      <c r="D67" s="135" t="s">
         <v>81</v>
       </c>
-      <c r="E67" s="130">
+      <c r="E67" s="103">
         <f>E66</f>
         <v>12.32</v>
       </c>
     </row>
     <row r="68" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B68" s="173">
+      <c r="B68" s="136">
         <v>6</v>
       </c>
-      <c r="C68" s="179" t="s">
+      <c r="C68" s="142" t="s">
         <v>53</v>
       </c>
-      <c r="D68" s="175" t="s">
+      <c r="D68" s="138" t="s">
         <v>78</v>
       </c>
-      <c r="E68" s="123">
+      <c r="E68" s="96">
         <v>5.67</v>
       </c>
-      <c r="F68" s="182">
+      <c r="F68" s="145">
         <f>E68</f>
         <v>5.67</v>
       </c>
     </row>
     <row r="69" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B69" s="170"/>
-      <c r="C69" s="180"/>
-      <c r="D69" s="172" t="s">
+      <c r="B69" s="133"/>
+      <c r="C69" s="143"/>
+      <c r="D69" s="135" t="s">
         <v>81</v>
       </c>
-      <c r="E69" s="130">
+      <c r="E69" s="103">
         <f>E68</f>
         <v>5.67</v>
       </c>
     </row>
     <row r="70" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B70" s="173">
+      <c r="B70" s="136">
         <v>7</v>
       </c>
-      <c r="C70" s="179" t="s">
-        <v>96</v>
-      </c>
-      <c r="D70" s="175" t="s">
+      <c r="C70" s="142" t="s">
+        <v>90</v>
+      </c>
+      <c r="D70" s="138" t="s">
         <v>78</v>
       </c>
-      <c r="E70" s="123">
+      <c r="E70" s="96">
         <v>12.01</v>
       </c>
-      <c r="F70" s="182">
+      <c r="F70" s="145">
         <f>E70</f>
         <v>12.01</v>
       </c>
     </row>
     <row r="71" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B71" s="170"/>
-      <c r="C71" s="180"/>
-      <c r="D71" s="172" t="s">
+      <c r="B71" s="133"/>
+      <c r="C71" s="143"/>
+      <c r="D71" s="135" t="s">
         <v>81</v>
       </c>
-      <c r="E71" s="130">
+      <c r="E71" s="103">
         <f>E70</f>
         <v>12.01</v>
       </c>
     </row>
     <row r="72" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B72" s="173">
+      <c r="B72" s="136">
         <v>8</v>
       </c>
-      <c r="C72" s="179" t="s">
-        <v>97</v>
-      </c>
-      <c r="D72" s="175" t="s">
+      <c r="C72" s="142" t="s">
+        <v>91</v>
+      </c>
+      <c r="D72" s="138" t="s">
         <v>78</v>
       </c>
-      <c r="E72" s="123">
+      <c r="E72" s="96">
         <v>17.239999999999998</v>
       </c>
-      <c r="F72" s="182">
+      <c r="F72" s="145">
         <f>E72</f>
         <v>17.239999999999998</v>
       </c>
     </row>
     <row r="73" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B73" s="170"/>
-      <c r="C73" s="180"/>
-      <c r="D73" s="172" t="s">
+      <c r="B73" s="133"/>
+      <c r="C73" s="143"/>
+      <c r="D73" s="135" t="s">
         <v>81</v>
       </c>
-      <c r="E73" s="130">
+      <c r="E73" s="103">
         <f>E72</f>
         <v>17.239999999999998</v>
       </c>
     </row>
     <row r="74" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B74" s="173">
+      <c r="B74" s="136">
         <v>9</v>
       </c>
-      <c r="C74" s="179" t="s">
+      <c r="C74" s="142" t="s">
         <v>56</v>
       </c>
-      <c r="D74" s="175" t="s">
+      <c r="D74" s="138" t="s">
         <v>78</v>
       </c>
-      <c r="E74" s="123">
+      <c r="E74" s="96">
         <v>192.38</v>
       </c>
     </row>
     <row r="75" spans="2:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B75" s="170"/>
-      <c r="C75" s="180"/>
-      <c r="D75" s="172" t="s">
+      <c r="B75" s="133"/>
+      <c r="C75" s="143"/>
+      <c r="D75" s="135" t="s">
         <v>81</v>
       </c>
-      <c r="E75" s="130">
+      <c r="E75" s="103">
         <f>E74</f>
         <v>192.38</v>
       </c>
     </row>
     <row r="76" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="F76" s="182">
+      <c r="F76" s="145">
         <f>SUM(F62:F73)</f>
         <v>196.33999999999997</v>
       </c>
     </row>
     <row r="78" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="F78" s="182">
+      <c r="F78" s="145">
         <f>F76-196.34</f>
         <v>0</v>
       </c>
@@ -5035,383 +5046,361 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:G28"/>
+  <dimension ref="A2:G23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.42578125" style="99" customWidth="1"/>
-    <col min="2" max="2" width="7.85546875" style="100" customWidth="1"/>
-    <col min="3" max="3" width="59.140625" style="99" customWidth="1"/>
-    <col min="4" max="4" width="10.7109375" style="101" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" style="109"/>
-    <col min="6" max="16384" width="9.140625" style="99"/>
+    <col min="1" max="1" width="6.42578125" style="76" customWidth="1"/>
+    <col min="2" max="2" width="7.85546875" style="77" customWidth="1"/>
+    <col min="3" max="3" width="53.85546875" style="76" customWidth="1"/>
+    <col min="4" max="4" width="9.140625" style="84"/>
+    <col min="5" max="5" width="14.5703125" style="68" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" style="78" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="76"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="110"/>
-      <c r="B3" s="111"/>
-      <c r="C3" s="143" t="s">
-        <v>91</v>
-      </c>
-      <c r="D3" s="112"/>
-      <c r="E3" s="113"/>
-      <c r="F3" s="114"/>
+      <c r="A3" s="85"/>
+      <c r="B3" s="86"/>
+      <c r="C3" s="114" t="s">
+        <v>86</v>
+      </c>
+      <c r="D3" s="88"/>
+      <c r="E3" s="70"/>
+      <c r="F3" s="87"/>
     </row>
     <row r="4" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="110"/>
-      <c r="B4" s="115" t="s">
+      <c r="A4" s="85"/>
+      <c r="B4" s="89" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="116" t="s">
+      <c r="C4" s="90" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="117" t="s">
+      <c r="D4" s="74" t="s">
+        <v>92</v>
+      </c>
+      <c r="E4" s="74" t="s">
+        <v>96</v>
+      </c>
+      <c r="F4" s="91" t="s">
         <v>68</v>
       </c>
-      <c r="E4" s="118"/>
-      <c r="F4" s="114"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="119"/>
-      <c r="B5" s="120">
-        <v>1</v>
-      </c>
-      <c r="C5" s="121" t="s">
-        <v>1</v>
-      </c>
-      <c r="D5" s="122">
+      <c r="A5" s="92"/>
+      <c r="B5" s="93">
+        <v>1</v>
+      </c>
+      <c r="C5" s="94" t="s">
+        <v>1</v>
+      </c>
+      <c r="D5" s="96" t="s">
+        <v>69</v>
+      </c>
+      <c r="E5" s="150">
+        <v>1</v>
+      </c>
+      <c r="F5" s="95">
         <f>G5</f>
         <v>2606.7700000000004</v>
       </c>
-      <c r="E5" s="123" t="s">
-        <v>69</v>
-      </c>
-      <c r="F5" s="114"/>
-      <c r="G5" s="99">
+      <c r="G5" s="76">
         <f>SUM('стены штукатурка'!H1:H75)</f>
         <v>2606.7700000000004</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="B6" s="107">
+      <c r="B6" s="82">
         <v>1.1000000000000001</v>
       </c>
-      <c r="C6" s="124" t="s">
+      <c r="C6" s="97" t="s">
         <v>73</v>
       </c>
-      <c r="D6" s="125">
+      <c r="D6" s="99" t="s">
+        <v>69</v>
+      </c>
+      <c r="E6" s="151">
+        <v>1</v>
+      </c>
+      <c r="F6" s="98">
         <v>991.77</v>
       </c>
-      <c r="E6" s="126" t="s">
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B7" s="82" t="s">
+        <v>61</v>
+      </c>
+      <c r="C7" s="100" t="s">
+        <v>60</v>
+      </c>
+      <c r="D7" s="99" t="s">
+        <v>72</v>
+      </c>
+      <c r="E7" s="151">
+        <v>1.3</v>
+      </c>
+      <c r="F7" s="98">
+        <f>F6*0.3</f>
+        <v>297.53100000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B8" s="82" t="s">
+        <v>62</v>
+      </c>
+      <c r="C8" s="100" t="s">
+        <v>75</v>
+      </c>
+      <c r="D8" s="99" t="s">
         <v>69</v>
       </c>
-      <c r="F6" s="114"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B7" s="107" t="s">
-        <v>61</v>
-      </c>
-      <c r="C7" s="127" t="s">
+      <c r="E8" s="151">
+        <f>E6*1.1</f>
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="F8" s="98">
+        <f>F6*1.1</f>
+        <v>1090.9470000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="83" t="s">
+        <v>63</v>
+      </c>
+      <c r="C9" s="101" t="s">
+        <v>71</v>
+      </c>
+      <c r="D9" s="103" t="s">
+        <v>72</v>
+      </c>
+      <c r="E9" s="151">
+        <v>1</v>
+      </c>
+      <c r="F9" s="102">
+        <f>F6*0.25</f>
+        <v>247.9425</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="93" t="s">
+        <v>64</v>
+      </c>
+      <c r="C10" s="104" t="s">
+        <v>74</v>
+      </c>
+      <c r="D10" s="96" t="s">
+        <v>69</v>
+      </c>
+      <c r="E10" s="152">
+        <f>E6*0.25</f>
+        <v>0.25</v>
+      </c>
+      <c r="F10" s="95">
+        <f>F5-F6</f>
+        <v>1615.0000000000005</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B11" s="82" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" s="100" t="s">
+        <v>76</v>
+      </c>
+      <c r="D11" s="99" t="s">
+        <v>72</v>
+      </c>
+      <c r="E11" s="157">
+        <v>1</v>
+      </c>
+      <c r="F11" s="98">
+        <f>F10*0.3</f>
+        <v>484.50000000000011</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="B12" s="82" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" s="100" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12" s="99" t="s">
+        <v>69</v>
+      </c>
+      <c r="E12" s="151">
+        <v>1.3</v>
+      </c>
+      <c r="F12" s="98">
+        <f>F10</f>
+        <v>1615.0000000000005</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="83" t="s">
+        <v>67</v>
+      </c>
+      <c r="C13" s="101" t="s">
         <v>60</v>
       </c>
-      <c r="D7" s="125">
-        <f>D6*1.3</f>
-        <v>1289.3009999999999</v>
-      </c>
-      <c r="E7" s="126" t="s">
+      <c r="D13" s="103" t="s">
         <v>72</v>
       </c>
-      <c r="F7" s="114"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B8" s="107" t="s">
-        <v>62</v>
-      </c>
-      <c r="C8" s="127" t="s">
-        <v>75</v>
-      </c>
-      <c r="D8" s="125">
-        <f>D6*1.1</f>
-        <v>1090.9470000000001</v>
-      </c>
-      <c r="E8" s="126" t="s">
+      <c r="E13" s="151">
+        <f>E11*1.1</f>
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="F13" s="102">
+        <f>F10*0.25</f>
+        <v>403.75000000000011</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="105">
+        <v>2</v>
+      </c>
+      <c r="C14" s="106" t="s">
+        <v>57</v>
+      </c>
+      <c r="D14" s="108" t="s">
         <v>69</v>
       </c>
-      <c r="F8" s="114"/>
-    </row>
-    <row r="9" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="108" t="s">
-        <v>63</v>
-      </c>
-      <c r="C9" s="128" t="s">
-        <v>71</v>
-      </c>
-      <c r="D9" s="129">
-        <f>D6*0.25</f>
-        <v>247.9425</v>
-      </c>
-      <c r="E9" s="130" t="s">
+      <c r="E14" s="151">
+        <v>1</v>
+      </c>
+      <c r="F14" s="107">
+        <f>F12+F8</f>
+        <v>2705.9470000000006</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="109">
+        <v>3</v>
+      </c>
+      <c r="C15" s="110" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="112" t="s">
+        <v>70</v>
+      </c>
+      <c r="E15" s="151">
+        <f>E11*0.15</f>
+        <v>0.15</v>
+      </c>
+      <c r="F15" s="111">
+        <v>717.45</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E16" s="153">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="80"/>
+      <c r="B18" s="165"/>
+      <c r="C18" s="166" t="s">
+        <v>87</v>
+      </c>
+      <c r="D18" s="167"/>
+      <c r="E18" s="168"/>
+      <c r="F18" s="166"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="80"/>
+      <c r="B19" s="165" t="s">
+        <v>6</v>
+      </c>
+      <c r="C19" s="169" t="s">
+        <v>7</v>
+      </c>
+      <c r="D19" s="170" t="s">
+        <v>92</v>
+      </c>
+      <c r="E19" s="170" t="s">
+        <v>96</v>
+      </c>
+      <c r="F19" s="171" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="80"/>
+      <c r="B20" s="172" t="s">
+        <v>82</v>
+      </c>
+      <c r="C20" s="169" t="s">
+        <v>78</v>
+      </c>
+      <c r="D20" s="98" t="s">
+        <v>69</v>
+      </c>
+      <c r="E20" s="151">
+        <v>1</v>
+      </c>
+      <c r="F20" s="79">
+        <v>1108.8800000000001</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="80"/>
+      <c r="B21" s="172" t="s">
+        <v>83</v>
+      </c>
+      <c r="C21" s="169" t="s">
+        <v>81</v>
+      </c>
+      <c r="D21" s="98" t="s">
+        <v>69</v>
+      </c>
+      <c r="E21" s="151">
+        <v>1</v>
+      </c>
+      <c r="F21" s="79">
+        <v>1108.8800000000001</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="80"/>
+      <c r="B22" s="172" t="s">
+        <v>84</v>
+      </c>
+      <c r="C22" s="173" t="s">
+        <v>80</v>
+      </c>
+      <c r="D22" s="98" t="s">
         <v>72</v>
       </c>
-      <c r="F9" s="114"/>
-    </row>
-    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="B10" s="120" t="s">
-        <v>64</v>
-      </c>
-      <c r="C10" s="131" t="s">
-        <v>74</v>
-      </c>
-      <c r="D10" s="122">
-        <f>D5-D6</f>
-        <v>1615.0000000000005</v>
-      </c>
-      <c r="E10" s="123" t="s">
-        <v>69</v>
-      </c>
-      <c r="F10" s="114"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B11" s="107" t="s">
-        <v>66</v>
-      </c>
-      <c r="C11" s="127" t="s">
-        <v>76</v>
-      </c>
-      <c r="D11" s="125">
-        <f>D10*1.3</f>
-        <v>2099.5000000000005</v>
-      </c>
-      <c r="E11" s="126" t="s">
+      <c r="E22" s="151">
+        <v>4.5</v>
+      </c>
+      <c r="F22" s="98">
+        <f>F21*4.5</f>
+        <v>4989.9600000000009</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B23" s="172" t="s">
+        <v>85</v>
+      </c>
+      <c r="C23" s="173" t="s">
+        <v>100</v>
+      </c>
+      <c r="D23" s="98" t="s">
         <v>72</v>
       </c>
-      <c r="F11" s="114"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B12" s="107" t="s">
-        <v>65</v>
-      </c>
-      <c r="C12" s="127" t="s">
-        <v>75</v>
-      </c>
-      <c r="D12" s="125">
-        <f>D10</f>
-        <v>1615.0000000000005</v>
-      </c>
-      <c r="E12" s="126" t="s">
-        <v>69</v>
-      </c>
-      <c r="F12" s="114"/>
-    </row>
-    <row r="13" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="108" t="s">
-        <v>67</v>
-      </c>
-      <c r="C13" s="128" t="s">
-        <v>60</v>
-      </c>
-      <c r="D13" s="129">
-        <f>D10*0.25</f>
-        <v>403.75000000000011</v>
-      </c>
-      <c r="E13" s="130" t="s">
-        <v>72</v>
-      </c>
-      <c r="F13" s="114"/>
-    </row>
-    <row r="14" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="132">
-        <v>2</v>
-      </c>
-      <c r="C14" s="133" t="s">
-        <v>57</v>
-      </c>
-      <c r="D14" s="134">
-        <f>D12+D8</f>
-        <v>2705.9470000000006</v>
-      </c>
-      <c r="E14" s="135" t="s">
-        <v>69</v>
-      </c>
-      <c r="F14" s="114"/>
-    </row>
-    <row r="15" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B15" s="136">
-        <v>3</v>
-      </c>
-      <c r="C15" s="137" t="s">
-        <v>11</v>
-      </c>
-      <c r="D15" s="138">
-        <v>717.45</v>
-      </c>
-      <c r="E15" s="139" t="s">
-        <v>70</v>
-      </c>
-      <c r="F15" s="114"/>
-    </row>
-    <row r="17" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="105"/>
-      <c r="B18" s="142"/>
-      <c r="C18" s="143" t="s">
-        <v>93</v>
-      </c>
-      <c r="D18" s="143"/>
-      <c r="E18" s="144"/>
-    </row>
-    <row r="19" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="105"/>
-      <c r="B19" s="115" t="s">
-        <v>6</v>
-      </c>
-      <c r="C19" s="148" t="s">
-        <v>7</v>
-      </c>
-      <c r="D19" s="117" t="s">
-        <v>68</v>
-      </c>
-      <c r="E19" s="151"/>
-    </row>
-    <row r="20" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="105"/>
-      <c r="B20" s="136" t="s">
-        <v>82</v>
-      </c>
-      <c r="C20" s="149" t="s">
-        <v>78</v>
-      </c>
-      <c r="D20" s="150">
-        <v>1268.4699999999998</v>
-      </c>
-      <c r="E20" s="139" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="105"/>
-      <c r="B21" s="120" t="s">
-        <v>83</v>
-      </c>
-      <c r="C21" s="145" t="s">
-        <v>1</v>
-      </c>
-      <c r="D21" s="146">
-        <v>58.519999999999996</v>
-      </c>
-      <c r="E21" s="123" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="105"/>
-      <c r="B22" s="107" t="s">
-        <v>84</v>
-      </c>
-      <c r="C22" s="140" t="s">
-        <v>76</v>
-      </c>
-      <c r="D22" s="103">
-        <f>D21*0.25</f>
-        <v>14.629999999999999</v>
-      </c>
-      <c r="E22" s="126" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="105"/>
-      <c r="B23" s="107" t="s">
-        <v>85</v>
-      </c>
-      <c r="C23" s="102" t="s">
-        <v>60</v>
-      </c>
-      <c r="D23" s="125">
-        <f>D21*0.15</f>
-        <v>8.7779999999999987</v>
-      </c>
-      <c r="E23" s="126" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="105"/>
-      <c r="B24" s="107" t="s">
-        <v>86</v>
-      </c>
-      <c r="C24" s="102" t="s">
-        <v>57</v>
-      </c>
-      <c r="D24" s="103">
-        <v>58.519999999999996</v>
-      </c>
-      <c r="E24" s="126" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="105"/>
-      <c r="B25" s="108" t="s">
-        <v>87</v>
-      </c>
-      <c r="C25" s="104" t="s">
-        <v>11</v>
-      </c>
-      <c r="D25" s="141">
-        <v>111.69</v>
-      </c>
-      <c r="E25" s="147" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="105"/>
-      <c r="B26" s="120" t="s">
-        <v>88</v>
-      </c>
-      <c r="C26" s="145" t="s">
-        <v>81</v>
-      </c>
-      <c r="D26" s="146">
-        <v>1268.4699999999998</v>
-      </c>
-      <c r="E26" s="123" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="105"/>
-      <c r="B27" s="107" t="s">
-        <v>89</v>
-      </c>
-      <c r="C27" s="102" t="s">
-        <v>80</v>
-      </c>
-      <c r="D27" s="125">
-        <f>D26*4.5</f>
-        <v>5708.1149999999989</v>
-      </c>
-      <c r="E27" s="126" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="108" t="s">
-        <v>90</v>
-      </c>
-      <c r="C28" s="104" t="s">
-        <v>92</v>
-      </c>
-      <c r="D28" s="129">
-        <f>D26*0.15</f>
-        <v>190.27049999999997</v>
-      </c>
-      <c r="E28" s="130" t="s">
-        <v>72</v>
+      <c r="E23" s="151">
+        <f>E21*0.15</f>
+        <v>0.15</v>
+      </c>
+      <c r="F23" s="98">
+        <f>F21*0.15</f>
+        <v>166.33200000000002</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>